<commit_message>
updated files in "annotated"
</commit_message>
<xml_diff>
--- a/annotators/team/tg/annotated/ted-mdb.1971.xlsx
+++ b/annotators/team/tg/annotated/ted-mdb.1971.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tabea\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tabea\Desktop\Git\AURIS\annotators\team\tg\annotated\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1345F7D3-5EB0-4B40-BBB3-F536E12560FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0CC5349-BFE0-49F7-B211-4C2672B6A120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1392" uniqueCount="512">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1368" uniqueCount="506">
   <si>
     <t>ID</t>
   </si>
@@ -1292,21 +1292,12 @@
     <t>sierra_leone</t>
   </si>
   <si>
-    <t>konkreter Ort</t>
-  </si>
-  <si>
     <t>westafrika</t>
   </si>
   <si>
-    <t>kein AUTO_REF</t>
-  </si>
-  <si>
     <t>90er</t>
   </si>
   <si>
-    <t>rebellenkrieg</t>
-  </si>
-  <si>
     <t>Antezedens</t>
   </si>
   <si>
@@ -1334,33 +1325,15 @@
     <t>OLD</t>
   </si>
   <si>
-    <t>bereits als GROUP etabliert</t>
-  </si>
-  <si>
-    <t>rebellenkrieg_angriff</t>
-  </si>
-  <si>
-    <t>Antezedens für folgenden Satz</t>
-  </si>
-  <si>
     <t>sprecher_kinder</t>
   </si>
   <si>
-    <t>krieg</t>
-  </si>
-  <si>
-    <t>amputationen</t>
-  </si>
-  <si>
     <t>menschen</t>
   </si>
   <si>
     <t>GEN</t>
   </si>
   <si>
-    <t>verwuestung</t>
-  </si>
-  <si>
     <t>amputierte_menschen</t>
   </si>
   <si>
@@ -1370,9 +1343,6 @@
     <t>prothesenschaft</t>
   </si>
   <si>
-    <t>stumpf</t>
-  </si>
-  <si>
     <t>prothese</t>
   </si>
   <si>
@@ -1385,9 +1355,6 @@
     <t>Teil der Verbvalenz</t>
   </si>
   <si>
-    <t>prothese_stelle</t>
-  </si>
-  <si>
     <t>PRED</t>
   </si>
   <si>
@@ -1397,9 +1364,6 @@
     <t>spezifische Untergruppe der amputierten Menschen</t>
   </si>
   <si>
-    <t>strategie_macht</t>
-  </si>
-  <si>
     <t>prothesenbauer</t>
   </si>
   <si>
@@ -1454,9 +1418,6 @@
     <t>druck</t>
   </si>
   <si>
-    <t>schmerzstelle</t>
-  </si>
-  <si>
     <t>Prothesenschäfte im Allgemeinen</t>
   </si>
   <si>
@@ -1466,48 +1427,15 @@
     <t>mit_mitarbeiter</t>
   </si>
   <si>
-    <t>versuch</t>
-  </si>
-  <si>
     <t>patient_veteran</t>
   </si>
   <si>
     <t>prothesen_mit</t>
   </si>
   <si>
-    <t>spezifische Untergruppe an Prothesen</t>
-  </si>
-  <si>
-    <t>CAT</t>
-  </si>
-  <si>
-    <t>leben_sinnvoll</t>
-  </si>
-  <si>
-    <t>Korrelat</t>
-  </si>
-  <si>
-    <t>werkzeuge</t>
-  </si>
-  <si>
-    <t>prozesse</t>
-  </si>
-  <si>
-    <t>werkzeuge+prozesse</t>
-  </si>
-  <si>
-    <t>Vorfeld-Platzhalter</t>
-  </si>
-  <si>
-    <t>materialien_prothesen</t>
-  </si>
-  <si>
     <t>Prothesen im Allgemeinen</t>
   </si>
   <si>
-    <t>krieg_betroffene</t>
-  </si>
-  <si>
     <t>boston</t>
   </si>
   <si>
@@ -1520,24 +1448,9 @@
     <t>doerfer_sierra</t>
   </si>
   <si>
-    <t>später Bezug auf diese Tätigkeit (substantiviert)</t>
-  </si>
-  <si>
-    <t>Antezedens; spezifischer Zeitpunkt; siehe log</t>
-  </si>
-  <si>
-    <t>AMBIG: auch GEN denkbar; allerdings spezifische Untergruppe an Menschen, die Sprecher kennt. Antezedens</t>
-  </si>
-  <si>
     <t>NEW</t>
   </si>
   <si>
-    <t>spezifische Untergruppe an Prothesen, die nicht passt und Druckschmerzen bereitet und erst später genauer beschrieben wird</t>
-  </si>
-  <si>
-    <t>syntaktischer Kopf; spezifische Untergruppe an Prothesenschäften, die zu Druckschmerz führen, hier beschrieben</t>
-  </si>
-  <si>
     <t>Antezedens; Problem der Nichtnutzung hier aufgemacht; siehe log</t>
   </si>
   <si>
@@ -1547,16 +1460,85 @@
     <t>AMBIG: SIT denkbar; allerdings handelt es sich um eine konkrete Forschungsgruppe der MIT Lab Mitarbeiter</t>
   </si>
   <si>
-    <t>belastungen</t>
-  </si>
-  <si>
     <t>auch ID mit_lab denkbar</t>
   </si>
   <si>
     <t>dieselbe Entität der Prothesen, die diese MIT Lab Gruppe herstellt</t>
   </si>
   <si>
-    <t>siehe log</t>
+    <t>brandschatzung</t>
+  </si>
+  <si>
+    <t>Antezedens für Temporaldeixis als Sprecher 12 Jahre alt war</t>
+  </si>
+  <si>
+    <t>parser error: syntaktisch gebundenes Relativpronomen</t>
+  </si>
+  <si>
+    <t>spezifische Untergruppe an Menschen, die Sprecher kennt; Antezedens</t>
+  </si>
+  <si>
+    <t>krieg_und_amputationen</t>
+  </si>
+  <si>
+    <t>Antezedens für "diese Verwüstung"</t>
+  </si>
+  <si>
+    <t>Bezug "Krieg und Amputationen" (GEN) wegen Dem.Pron. Gewählt</t>
+  </si>
+  <si>
+    <t>spezifische Untergruppe an Prothesen, die nicht passt, Druckschmerzen bereitet und erst später genauer beschrieben wird</t>
+  </si>
+  <si>
+    <t>spezifische Untergruppe an Prothesenschäften, die zu Druckschmerz führen</t>
+  </si>
+  <si>
+    <t>"Knöchel"prothese unklar</t>
+  </si>
+  <si>
+    <t>doktorarbeit_sprecher</t>
+  </si>
+  <si>
+    <t>usa</t>
+  </si>
+  <si>
+    <t>zwar nicht syntaktischer Kopf, aber Bezug konkrete lokale Entität</t>
+  </si>
+  <si>
+    <t>syntaktisch gebundenes Korrelat</t>
+  </si>
+  <si>
+    <t>hoffnung_sprecher</t>
+  </si>
+  <si>
+    <t>parser error nach Pos.Pron.</t>
+  </si>
+  <si>
+    <t>werkzeuge_und_prozesse</t>
+  </si>
+  <si>
+    <t>mit_gruppe</t>
+  </si>
+  <si>
+    <t>seelen_betroffener</t>
+  </si>
+  <si>
+    <t>REF=OLD, weil als GROUP etabliert</t>
+  </si>
+  <si>
+    <t>Antezedens für folgende solcher Angriffe</t>
+  </si>
+  <si>
+    <t>patient_glieder</t>
+  </si>
+  <si>
+    <t>glauben_patient</t>
+  </si>
+  <si>
+    <t>parser error: Relativpronomen</t>
+  </si>
+  <si>
+    <t>parser error nach Pos.Pron.; spezifische Untergruppe an Prothesen</t>
   </si>
 </sst>
 </file>
@@ -2256,7 +2238,7 @@
         <v>38</v>
       </c>
       <c r="E4" s="21" t="str">
-        <f t="shared" ref="E3:E66" si="1">IF(D4="?OLD","!!!","")</f>
+        <f t="shared" ref="E4:E66" si="1">IF(D4="?OLD","!!!","")</f>
         <v/>
       </c>
       <c r="F4" s="22" t="str">
@@ -2359,9 +2341,7 @@
         <f>IF(OR(E6="",E6="!!!",F6="NEW"),"",INDEX(J$1:J5,SUMPRODUCT(MAX(ROW(E$1:E5)*(E6=E$1:E5)))))</f>
         <v/>
       </c>
-      <c r="L6" s="26" t="s">
-        <v>423</v>
-      </c>
+      <c r="L6" s="26"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -2713,16 +2693,14 @@
       <c r="C17" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="E17" s="21" t="s">
-        <v>422</v>
-      </c>
+      <c r="E17" s="21"/>
       <c r="F17" s="22" t="str">
         <f>IF(OR(E17="",E17="!!!"),"",IF(NOT(ISNA(VLOOKUP(E17,E$1:E16,1,FALSE()))),"OLD",IF(AND(E17&lt;&gt;"",E17&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v/>
       </c>
       <c r="G17" s="23" t="str">
-        <f ca="1">IF(OR(E17="",E17="!!!"),"",IF(OR(J17=0,AND(J17=1,K17=1),AND(J17=1,I17="SBJ"),AND(J17=1,I17=0)),"?IN_FOCUS",IF(J17&lt;=2,"?ACTIVATED",IF(J17&lt;&gt;"","?FAMILIAR",IF(F17="NEW",IF(ISNA(VLOOKUP(E17,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E17="",E17="!!!"),"",IF(OR(J17=0,AND(J17=1,K17=1),AND(J17=1,I17="SBJ"),AND(J17=1,I17=0)),"?IN_FOCUS",IF(J17&lt;=2,"?ACTIVATED",IF(J17&lt;&gt;"","?FAMILIAR",IF(F17="NEW",IF(ISNA(VLOOKUP(E17,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H17" s="24" t="str">
         <f t="shared" ca="1" si="0"/>
@@ -2730,19 +2708,17 @@
       </c>
       <c r="I17" s="25" t="str">
         <f>IF(OR(E17="",E17="!!!",F17="NEW"),"",INDEX(B$2:B16,-1+SUMPRODUCT(MAX(ROW(E$2:E16)*(E17=E$2:E16)))))</f>
-        <v>other_2</v>
-      </c>
-      <c r="J17" s="25">
+        <v/>
+      </c>
+      <c r="J17" s="25" t="str">
         <f ca="1">IF(OR(E17="",E17="!!!",F17="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E17)*(E17=E$2:E17)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E16)*(E2=E$1:E16))))))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K17" s="25" t="str">
-        <f ca="1">IF(OR(E17="",E17="!!!",F17="NEW"),"",INDEX(J$1:J16,SUMPRODUCT(MAX(ROW(E$1:E16)*(E17=E$1:E16)))))</f>
-        <v/>
-      </c>
-      <c r="L17" s="26" t="s">
-        <v>425</v>
-      </c>
+        <f>IF(OR(E17="",E17="!!!",F17="NEW"),"",INDEX(J$1:J16,SUMPRODUCT(MAX(ROW(E$1:E16)*(E17=E$1:E16)))))</f>
+        <v/>
+      </c>
+      <c r="L17" s="26"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
@@ -2792,7 +2768,7 @@
         <v>37</v>
       </c>
       <c r="E19" s="21" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="F19" s="22" t="str">
         <f>IF(OR(E19="",E19="!!!"),"",IF(NOT(ISNA(VLOOKUP(E19,E$1:E18,1,FALSE()))),"OLD",IF(AND(E19&lt;&gt;"",E19&lt;&gt;"!!!"),"NEW","")))</f>
@@ -2898,16 +2874,14 @@
       <c r="C22" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="E22" s="21" t="s">
-        <v>422</v>
-      </c>
+      <c r="E22" s="21"/>
       <c r="F22" s="22" t="str">
         <f>IF(OR(E22="",E22="!!!"),"",IF(NOT(ISNA(VLOOKUP(E22,E$1:E21,1,FALSE()))),"OLD",IF(AND(E22&lt;&gt;"",E22&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v/>
       </c>
       <c r="G22" s="23" t="str">
-        <f ca="1">IF(OR(E22="",E22="!!!"),"",IF(OR(J22=0,AND(J22=1,K22=1),AND(J22=1,I22="SBJ"),AND(J22=1,I22=0)),"?IN_FOCUS",IF(J22&lt;=2,"?ACTIVATED",IF(J22&lt;&gt;"","?FAMILIAR",IF(F22="NEW",IF(ISNA(VLOOKUP(E22,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E22="",E22="!!!"),"",IF(OR(J22=0,AND(J22=1,K22=1),AND(J22=1,I22="SBJ"),AND(J22=1,I22=0)),"?IN_FOCUS",IF(J22&lt;=2,"?ACTIVATED",IF(J22&lt;&gt;"","?FAMILIAR",IF(F22="NEW",IF(ISNA(VLOOKUP(E22,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H22" s="24" t="str">
         <f t="shared" ca="1" si="0"/>
@@ -2915,19 +2889,17 @@
       </c>
       <c r="I22" s="25" t="str">
         <f>IF(OR(E22="",E22="!!!",F22="NEW"),"",INDEX(B$2:B21,-1+SUMPRODUCT(MAX(ROW(E$2:E21)*(E22=E$2:E21)))))</f>
-        <v>other_3</v>
-      </c>
-      <c r="J22" s="25">
+        <v/>
+      </c>
+      <c r="J22" s="25" t="str">
         <f ca="1">IF(OR(E22="",E22="!!!",F22="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E22)*(E22=E$2:E22)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E21)*(E2=E$1:E21))))))</f>
-        <v>0</v>
-      </c>
-      <c r="K22" s="25">
-        <f ca="1">IF(OR(E22="",E22="!!!",F22="NEW"),"",INDEX(J$1:J21,SUMPRODUCT(MAX(ROW(E$1:E21)*(E22=E$1:E21)))))</f>
-        <v>0</v>
-      </c>
-      <c r="L22" s="26" t="s">
-        <v>425</v>
-      </c>
+        <v/>
+      </c>
+      <c r="K22" s="25" t="str">
+        <f>IF(OR(E22="",E22="!!!",F22="NEW"),"",INDEX(J$1:J21,SUMPRODUCT(MAX(ROW(E$1:E21)*(E22=E$1:E21)))))</f>
+        <v/>
+      </c>
+      <c r="L22" s="26"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
@@ -3379,15 +3351,15 @@
       </c>
       <c r="I35" s="25" t="str">
         <f>IF(OR(E35="",E35="!!!",F35="NEW"),"",INDEX(B$2:B34,-1+SUMPRODUCT(MAX(ROW(E$2:E34)*(E35=E$2:E34)))))</f>
-        <v>other_5</v>
+        <v>other_2</v>
       </c>
       <c r="J35" s="25">
         <f ca="1">IF(OR(E35="",E35="!!!",F35="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E35)*(E35=E$2:E35)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E34)*(E2=E$1:E34))))))</f>
         <v>0</v>
       </c>
-      <c r="K35" s="25">
+      <c r="K35" s="25" t="str">
         <f ca="1">IF(OR(E35="",E35="!!!",F35="NEW"),"",INDEX(J$1:J34,SUMPRODUCT(MAX(ROW(E$1:E34)*(E35=E$1:E34)))))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="L35" s="26"/>
     </row>
@@ -3571,16 +3543,14 @@
       <c r="C41" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="E41" s="21" t="s">
-        <v>427</v>
-      </c>
+      <c r="E41" s="21"/>
       <c r="F41" s="22" t="str">
         <f>IF(OR(E41="",E41="!!!"),"",IF(NOT(ISNA(VLOOKUP(E41,E$1:E40,1,FALSE()))),"OLD",IF(AND(E41&lt;&gt;"",E41&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>NEW</v>
+        <v/>
       </c>
       <c r="G41" s="23" t="str">
-        <f ca="1">IF(OR(E41="",E41="!!!"),"",IF(OR(J41=0,AND(J41=1,K41=1),AND(J41=1,I41="SBJ"),AND(J41=1,I41=0)),"?IN_FOCUS",IF(J41&lt;=2,"?ACTIVATED",IF(J41&lt;&gt;"","?FAMILIAR",IF(F41="NEW",IF(ISNA(VLOOKUP(E41,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?REFERENTIAL</v>
+        <f>IF(OR(E41="",E41="!!!"),"",IF(OR(J41=0,AND(J41=1,K41=1),AND(J41=1,I41="SBJ"),AND(J41=1,I41=0)),"?IN_FOCUS",IF(J41&lt;=2,"?ACTIVATED",IF(J41&lt;&gt;"","?FAMILIAR",IF(F41="NEW",IF(ISNA(VLOOKUP(E41,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H41" s="24" t="str">
         <f t="shared" ca="1" si="0"/>
@@ -3598,9 +3568,7 @@
         <f>IF(OR(E41="",E41="!!!",F41="NEW"),"",INDEX(J$1:J40,SUMPRODUCT(MAX(ROW(E$1:E40)*(E41=E$1:E40)))))</f>
         <v/>
       </c>
-      <c r="L41" s="26" t="s">
-        <v>428</v>
-      </c>
+      <c r="L41" s="26"/>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
@@ -3684,7 +3652,7 @@
         <v>37</v>
       </c>
       <c r="E44" s="21" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="F44" s="22" t="str">
         <f>IF(OR(E44="",E44="!!!"),"",IF(NOT(ISNA(VLOOKUP(E44,E$1:E43,1,FALSE()))),"OLD",IF(AND(E44&lt;&gt;"",E44&lt;&gt;"!!!"),"NEW","")))</f>
@@ -3711,7 +3679,7 @@
         <v/>
       </c>
       <c r="L44" s="26" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.3">
@@ -3786,16 +3754,14 @@
       <c r="A47" t="s">
         <v>79</v>
       </c>
-      <c r="E47" s="21" t="s">
-        <v>427</v>
-      </c>
+      <c r="E47" s="21"/>
       <c r="F47" s="22" t="str">
         <f>IF(OR(E47="",E47="!!!"),"",IF(NOT(ISNA(VLOOKUP(E47,E$1:E46,1,FALSE()))),"OLD",IF(AND(E47&lt;&gt;"",E47&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v/>
       </c>
       <c r="G47" s="23" t="str">
-        <f ca="1">IF(OR(E47="",E47="!!!"),"",IF(OR(J47=0,AND(J47=1,K47=1),AND(J47=1,I47="SBJ"),AND(J47=1,I47=0)),"?IN_FOCUS",IF(J47&lt;=2,"?ACTIVATED",IF(J47&lt;&gt;"","?FAMILIAR",IF(F47="NEW",IF(ISNA(VLOOKUP(E47,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E47="",E47="!!!"),"",IF(OR(J47=0,AND(J47=1,K47=1),AND(J47=1,I47="SBJ"),AND(J47=1,I47=0)),"?IN_FOCUS",IF(J47&lt;=2,"?ACTIVATED",IF(J47&lt;&gt;"","?FAMILIAR",IF(F47="NEW",IF(ISNA(VLOOKUP(E47,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H47" s="24" t="str">
         <f t="shared" ca="1" si="0"/>
@@ -3803,19 +3769,17 @@
       </c>
       <c r="I47" s="25" t="str">
         <f>IF(OR(E47="",E47="!!!",F47="NEW"),"",INDEX(B$2:B46,-1+SUMPRODUCT(MAX(ROW(E$2:E46)*(E47=E$2:E46)))))</f>
-        <v>other_3</v>
-      </c>
-      <c r="J47" s="25">
+        <v/>
+      </c>
+      <c r="J47" s="25" t="str">
         <f ca="1">IF(OR(E47="",E47="!!!",F47="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E47)*(E47=E$2:E47)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E46)*(E2=E$1:E46))))))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K47" s="25" t="str">
-        <f ca="1">IF(OR(E47="",E47="!!!",F47="NEW"),"",INDEX(J$1:J46,SUMPRODUCT(MAX(ROW(E$1:E46)*(E47=E$1:E46)))))</f>
-        <v/>
-      </c>
-      <c r="L47" s="26" t="s">
-        <v>425</v>
-      </c>
+        <f>IF(OR(E47="",E47="!!!",F47="NEW"),"",INDEX(J$1:J46,SUMPRODUCT(MAX(ROW(E$1:E46)*(E47=E$1:E46)))))</f>
+        <v/>
+      </c>
+      <c r="L47" s="26"/>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
@@ -3865,7 +3829,7 @@
         <v>37</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>498</v>
+        <v>474</v>
       </c>
       <c r="F49" s="22" t="str">
         <f>IF(OR(E49="",E49="!!!"),"",IF(NOT(ISNA(VLOOKUP(E49,E$1:E48,1,FALSE()))),"OLD",IF(AND(E49&lt;&gt;"",E49&lt;&gt;"!!!"),"NEW","")))</f>
@@ -3897,17 +3861,16 @@
       <c r="A50" t="s">
         <v>82</v>
       </c>
-      <c r="E50" s="21" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+      <c r="E50" s="21" t="s">
+        <v>481</v>
       </c>
       <c r="F50" s="22" t="str">
         <f>IF(OR(E50="",E50="!!!"),"",IF(NOT(ISNA(VLOOKUP(E50,E$1:E49,1,FALSE()))),"OLD",IF(AND(E50&lt;&gt;"",E50&lt;&gt;"!!!"),"NEW","")))</f>
-        <v/>
+        <v>NEW</v>
       </c>
       <c r="G50" s="23" t="str">
-        <f>IF(OR(E50="",E50="!!!"),"",IF(OR(J50=0,AND(J50=1,K50=1),AND(J50=1,I50="SBJ"),AND(J50=1,I50=0)),"?IN_FOCUS",IF(J50&lt;=2,"?ACTIVATED",IF(J50&lt;&gt;"","?FAMILIAR",IF(F50="NEW",IF(ISNA(VLOOKUP(E50,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v/>
+        <f ca="1">IF(OR(E50="",E50="!!!"),"",IF(OR(J50=0,AND(J50=1,K50=1),AND(J50=1,I50="SBJ"),AND(J50=1,I50=0)),"?IN_FOCUS",IF(J50&lt;=2,"?ACTIVATED",IF(J50&lt;&gt;"","?FAMILIAR",IF(F50="NEW",IF(ISNA(VLOOKUP(E50,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v>?REFERENTIAL</v>
       </c>
       <c r="H50" s="24" t="str">
         <f t="shared" ca="1" si="0"/>
@@ -3925,7 +3888,9 @@
         <f>IF(OR(E50="",E50="!!!",F50="NEW"),"",INDEX(J$1:J49,SUMPRODUCT(MAX(ROW(E$1:E49)*(E50=E$1:E49)))))</f>
         <v/>
       </c>
-      <c r="L50" s="26"/>
+      <c r="L50" s="26" t="s">
+        <v>501</v>
+      </c>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
@@ -4392,7 +4357,7 @@
         <v/>
       </c>
       <c r="L63" s="26" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.3">
@@ -4409,7 +4374,7 @@
         <v>37</v>
       </c>
       <c r="E64" s="21" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="F64" s="22" t="str">
         <f>IF(OR(E64="",E64="!!!"),"",IF(NOT(ISNA(VLOOKUP(E64,E$1:E63,1,FALSE()))),"OLD",IF(AND(E64&lt;&gt;"",E64&lt;&gt;"!!!"),"NEW","")))</f>
@@ -4555,16 +4520,14 @@
       <c r="A68" t="s">
         <v>98</v>
       </c>
-      <c r="E68" s="21" t="s">
-        <v>442</v>
-      </c>
+      <c r="E68" s="21"/>
       <c r="F68" s="22" t="str">
         <f>IF(OR(E68="",E68="!!!"),"",IF(NOT(ISNA(VLOOKUP(E68,E$1:E67,1,FALSE()))),"OLD",IF(AND(E68&lt;&gt;"",E68&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>NEW</v>
+        <v/>
       </c>
       <c r="G68" s="23" t="str">
-        <f ca="1">IF(OR(E68="",E68="!!!"),"",IF(OR(J68=0,AND(J68=1,K68=1),AND(J68=1,I68="SBJ"),AND(J68=1,I68=0)),"?IN_FOCUS",IF(J68&lt;=2,"?ACTIVATED",IF(J68&lt;&gt;"","?FAMILIAR",IF(F68="NEW",IF(ISNA(VLOOKUP(E68,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?REFERENTIAL</v>
+        <f>IF(OR(E68="",E68="!!!"),"",IF(OR(J68=0,AND(J68=1,K68=1),AND(J68=1,I68="SBJ"),AND(J68=1,I68=0)),"?IN_FOCUS",IF(J68&lt;=2,"?ACTIVATED",IF(J68&lt;&gt;"","?FAMILIAR",IF(F68="NEW",IF(ISNA(VLOOKUP(E68,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H68" s="24" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -4582,9 +4545,7 @@
         <f>IF(OR(E68="",E68="!!!",F68="NEW"),"",INDEX(J$1:J67,SUMPRODUCT(MAX(ROW(E$1:E67)*(E68=E$1:E67)))))</f>
         <v/>
       </c>
-      <c r="L68" s="26" t="s">
-        <v>499</v>
-      </c>
+      <c r="L68" s="26"/>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
@@ -4673,7 +4634,7 @@
         <v>62</v>
       </c>
       <c r="E71" s="21" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="F71" s="22" t="str">
         <f>IF(OR(E71="",E71="!!!"),"",IF(NOT(ISNA(VLOOKUP(E71,E$1:E70,1,FALSE()))),"OLD",IF(AND(E71&lt;&gt;"",E71&lt;&gt;"!!!"),"NEW","")))</f>
@@ -4777,39 +4738,39 @@
       </c>
       <c r="L73" s="26"/>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>103</v>
       </c>
-      <c r="E74" s="21" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="F74" s="22" t="str">
-        <f>IF(OR(E74="",E74="!!!"),"",IF(NOT(ISNA(VLOOKUP(E74,E$1:E73,1,FALSE()))),"OLD",IF(AND(E74&lt;&gt;"",E74&lt;&gt;"!!!"),"NEW","")))</f>
-        <v/>
-      </c>
-      <c r="G74" s="23" t="str">
-        <f>IF(OR(E74="",E74="!!!"),"",IF(OR(J74=0,AND(J74=1,K74=1),AND(J74=1,I74="SBJ"),AND(J74=1,I74=0)),"?IN_FOCUS",IF(J74&lt;=2,"?ACTIVATED",IF(J74&lt;&gt;"","?FAMILIAR",IF(F74="NEW",IF(ISNA(VLOOKUP(E74,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v/>
+      <c r="E74" s="21" t="s">
+        <v>431</v>
+      </c>
+      <c r="F74" s="22" t="s">
+        <v>419</v>
+      </c>
+      <c r="G74" s="23" t="e">
+        <f ca="1">IF(OR(E74="",E74="!!!"),"",IF(OR(J74=0,AND(J74=1,K74=1),AND(J74=1,I74="SBJ"),AND(J74=1,I74=0)),"?IN_FOCUS",IF(J74&lt;=2,"?ACTIVATED",IF(J74&lt;&gt;"","?FAMILIAR",IF(F74="NEW",IF(ISNA(VLOOKUP(E74,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v>#VALUE!</v>
       </c>
       <c r="H74" s="24" t="str">
         <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="I74" s="25" t="str">
+      <c r="I74" s="25" t="e">
         <f>IF(OR(E74="",E74="!!!",F74="NEW"),"",INDEX(B$2:B73,-1+SUMPRODUCT(MAX(ROW(E$2:E73)*(E74=E$2:E73)))))</f>
-        <v/>
-      </c>
-      <c r="J74" s="25" t="str">
+        <v>#VALUE!</v>
+      </c>
+      <c r="J74" s="25">
         <f ca="1">IF(OR(E74="",E74="!!!",F74="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E74)*(E74=E$2:E74)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E73)*(E2=E$1:E73))))))</f>
-        <v/>
-      </c>
-      <c r="K74" s="25" t="str">
+        <v>0</v>
+      </c>
+      <c r="K74" s="25" t="e">
         <f>IF(OR(E74="",E74="!!!",F74="NEW"),"",INDEX(J$1:J73,SUMPRODUCT(MAX(ROW(E$1:E73)*(E74=E$1:E73)))))</f>
-        <v/>
-      </c>
-      <c r="L74" s="26"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L74" s="26" t="s">
+        <v>482</v>
+      </c>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
@@ -4825,10 +4786,10 @@
         <v>37</v>
       </c>
       <c r="E75" s="21" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="F75" s="22" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="G75" s="23" t="e">
         <f ca="1">IF(OR(E75="",E75="!!!"),"",IF(OR(J75=0,AND(J75=1,K75=1),AND(J75=1,I75="SBJ"),AND(J75=1,I75=0)),"?IN_FOCUS",IF(J75&lt;=2,"?ACTIVATED",IF(J75&lt;&gt;"","?FAMILIAR",IF(F75="NEW",IF(ISNA(VLOOKUP(E75,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
@@ -4890,16 +4851,14 @@
       <c r="A77" t="s">
         <v>48</v>
       </c>
-      <c r="E77" s="21" t="s">
-        <v>438</v>
-      </c>
+      <c r="E77" s="21"/>
       <c r="F77" s="22" t="str">
         <f>IF(OR(E77="",E77="!!!"),"",IF(NOT(ISNA(VLOOKUP(E77,E$1:E76,1,FALSE()))),"OLD",IF(AND(E77&lt;&gt;"",E77&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>NEW</v>
+        <v/>
       </c>
       <c r="G77" s="23" t="str">
-        <f ca="1">IF(OR(E77="",E77="!!!"),"",IF(OR(J77=0,AND(J77=1,K77=1),AND(J77=1,I77="SBJ"),AND(J77=1,I77=0)),"?IN_FOCUS",IF(J77&lt;=2,"?ACTIVATED",IF(J77&lt;&gt;"","?FAMILIAR",IF(F77="NEW",IF(ISNA(VLOOKUP(E77,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?REFERENTIAL</v>
+        <f>IF(OR(E77="",E77="!!!"),"",IF(OR(J77=0,AND(J77=1,K77=1),AND(J77=1,I77="SBJ"),AND(J77=1,I77=0)),"?IN_FOCUS",IF(J77&lt;=2,"?ACTIVATED",IF(J77&lt;&gt;"","?FAMILIAR",IF(F77="NEW",IF(ISNA(VLOOKUP(E77,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H77" s="24" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -4917,9 +4876,7 @@
         <f>IF(OR(E77="",E77="!!!",F77="NEW"),"",INDEX(J$1:J76,SUMPRODUCT(MAX(ROW(E$1:E76)*(E77=E$1:E76)))))</f>
         <v/>
       </c>
-      <c r="L77" s="26" t="s">
-        <v>439</v>
-      </c>
+      <c r="L77" s="26"/>
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
@@ -4960,7 +4917,7 @@
         <v/>
       </c>
       <c r="L78" s="26" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.3">
@@ -4977,7 +4934,7 @@
         <v>37</v>
       </c>
       <c r="E79" s="21" t="s">
-        <v>427</v>
+        <v>481</v>
       </c>
       <c r="F79" s="22" t="str">
         <f>IF(OR(E79="",E79="!!!"),"",IF(NOT(ISNA(VLOOKUP(E79,E$1:E78,1,FALSE()))),"OLD",IF(AND(E79&lt;&gt;"",E79&lt;&gt;"!!!"),"NEW","")))</f>
@@ -4999,9 +4956,9 @@
         <f ca="1">IF(OR(E79="",E79="!!!",F79="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E79)*(E79=E$2:E79)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E78)*(E2=E$1:E78))))))</f>
         <v>0</v>
       </c>
-      <c r="K79" s="25">
+      <c r="K79" s="25" t="str">
         <f ca="1">IF(OR(E79="",E79="!!!",F79="NEW"),"",INDEX(J$1:J78,SUMPRODUCT(MAX(ROW(E$1:E78)*(E79=E$1:E78)))))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="L79" s="26"/>
     </row>
@@ -5117,35 +5074,29 @@
       <c r="A83" t="s">
         <v>63</v>
       </c>
-      <c r="E83" s="21" t="s">
-        <v>434</v>
-      </c>
-      <c r="F83" s="22" t="s">
-        <v>419</v>
-      </c>
-      <c r="G83" s="23" t="e">
-        <f ca="1">IF(OR(E83="",E83="!!!"),"",IF(OR(J83=0,AND(J83=1,K83=1),AND(J83=1,I83="SBJ"),AND(J83=1,I83=0)),"?IN_FOCUS",IF(J83&lt;=2,"?ACTIVATED",IF(J83&lt;&gt;"","?FAMILIAR",IF(F83="NEW",IF(ISNA(VLOOKUP(E83,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>#VALUE!</v>
+      <c r="E83" s="21"/>
+      <c r="F83" s="22"/>
+      <c r="G83" s="23" t="str">
+        <f>IF(OR(E83="",E83="!!!"),"",IF(OR(J83=0,AND(J83=1,K83=1),AND(J83=1,I83="SBJ"),AND(J83=1,I83=0)),"?IN_FOCUS",IF(J83&lt;=2,"?ACTIVATED",IF(J83&lt;&gt;"","?FAMILIAR",IF(F83="NEW",IF(ISNA(VLOOKUP(E83,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H83" s="24" t="str">
         <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="I83" s="25" t="e">
+      <c r="I83" s="25" t="str">
         <f>IF(OR(E83="",E83="!!!",F83="NEW"),"",INDEX(B$2:B82,-1+SUMPRODUCT(MAX(ROW(E$2:E82)*(E83=E$2:E82)))))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="J83" s="25">
+        <v/>
+      </c>
+      <c r="J83" s="25" t="str">
         <f ca="1">IF(OR(E83="",E83="!!!",F83="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E83)*(E83=E$2:E83)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E82)*(E2=E$1:E82))))))</f>
-        <v>0</v>
-      </c>
-      <c r="K83" s="25" t="e">
+        <v/>
+      </c>
+      <c r="K83" s="25" t="str">
         <f>IF(OR(E83="",E83="!!!",F83="NEW"),"",INDEX(J$1:J82,SUMPRODUCT(MAX(ROW(E$1:E82)*(E83=E$1:E82)))))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L83" s="26" t="s">
-        <v>500</v>
-      </c>
+        <v/>
+      </c>
+      <c r="L83" s="26"/>
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
@@ -5364,7 +5315,7 @@
         <v/>
       </c>
       <c r="L89" s="26" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.3">
@@ -5381,7 +5332,7 @@
         <v>37</v>
       </c>
       <c r="E90" s="21" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="F90" s="22" t="str">
         <f>IF(OR(E90="",E90="!!!"),"",IF(NOT(ISNA(VLOOKUP(E90,E$1:E89,1,FALSE()))),"OLD",IF(AND(E90&lt;&gt;"",E90&lt;&gt;"!!!"),"NEW","")))</f>
@@ -5519,7 +5470,9 @@
         <f ca="1">IF(OR(E93="",E93="!!!",F93="NEW"),"",INDEX(J$1:J92,SUMPRODUCT(MAX(ROW(E$1:E92)*(E93=E$1:E92)))))</f>
         <v>0</v>
       </c>
-      <c r="L93" s="26"/>
+      <c r="L93" s="26" t="s">
+        <v>455</v>
+      </c>
     </row>
     <row r="94" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
@@ -5954,7 +5907,7 @@
         <v>62</v>
       </c>
       <c r="E106" s="21" t="s">
-        <v>440</v>
+        <v>434</v>
       </c>
       <c r="F106" s="22" t="str">
         <f>IF(OR(E106="",E106="!!!"),"",IF(NOT(ISNA(VLOOKUP(E106,E$1:E105,1,FALSE()))),"OLD",IF(AND(E106&lt;&gt;"",E106&lt;&gt;"!!!"),"NEW","")))</f>
@@ -5981,7 +5934,7 @@
         <v/>
       </c>
       <c r="L106" s="26" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
     </row>
     <row r="107" spans="1:12" x14ac:dyDescent="0.3">
@@ -6026,7 +5979,7 @@
         <v>35</v>
       </c>
       <c r="E108" s="21" t="s">
-        <v>438</v>
+        <v>481</v>
       </c>
       <c r="F108" s="22" t="str">
         <f>IF(OR(E108="",E108="!!!"),"",IF(NOT(ISNA(VLOOKUP(E108,E$1:E107,1,FALSE()))),"OLD",IF(AND(E108&lt;&gt;"",E108&lt;&gt;"!!!"),"NEW","")))</f>
@@ -6040,17 +5993,17 @@
         <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="I108" s="25">
+      <c r="I108" s="25" t="str">
         <f>IF(OR(E108="",E108="!!!",F108="NEW"),"",INDEX(B$2:B107,-1+SUMPRODUCT(MAX(ROW(E$2:E107)*(E108=E$2:E107)))))</f>
-        <v>0</v>
+        <v>other_3</v>
       </c>
       <c r="J108" s="25">
         <f ca="1">IF(OR(E108="",E108="!!!",F108="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E108)*(E108=E$2:E108)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E107)*(E2=E$1:E107))))))</f>
         <v>0</v>
       </c>
-      <c r="K108" s="25" t="str">
+      <c r="K108" s="25">
         <f ca="1">IF(OR(E108="",E108="!!!",F108="NEW"),"",INDEX(J$1:J107,SUMPRODUCT(MAX(ROW(E$1:E107)*(E108=E$1:E107)))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L108" s="26"/>
     </row>
@@ -6156,7 +6109,7 @@
       </c>
       <c r="L111" s="26"/>
     </row>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>134</v>
       </c>
@@ -6169,16 +6122,14 @@
       <c r="D112" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="E112" s="21" t="s">
-        <v>438</v>
-      </c>
+      <c r="E112" s="21"/>
       <c r="F112" s="22" t="str">
         <f>IF(OR(E112="",E112="!!!"),"",IF(NOT(ISNA(VLOOKUP(E112,E$1:E111,1,FALSE()))),"OLD",IF(AND(E112&lt;&gt;"",E112&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v/>
       </c>
       <c r="G112" s="23" t="str">
-        <f ca="1">IF(OR(E112="",E112="!!!"),"",IF(OR(J112=0,AND(J112=1,K112=1),AND(J112=1,I112="SBJ"),AND(J112=1,I112=0)),"?IN_FOCUS",IF(J112&lt;=2,"?ACTIVATED",IF(J112&lt;&gt;"","?FAMILIAR",IF(F112="NEW",IF(ISNA(VLOOKUP(E112,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E112="",E112="!!!"),"",IF(OR(J112=0,AND(J112=1,K112=1),AND(J112=1,I112="SBJ"),AND(J112=1,I112=0)),"?IN_FOCUS",IF(J112&lt;=2,"?ACTIVATED",IF(J112&lt;&gt;"","?FAMILIAR",IF(F112="NEW",IF(ISNA(VLOOKUP(E112,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H112" s="24" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -6186,17 +6137,19 @@
       </c>
       <c r="I112" s="25" t="str">
         <f>IF(OR(E112="",E112="!!!",F112="NEW"),"",INDEX(B$2:B111,-1+SUMPRODUCT(MAX(ROW(E$2:E111)*(E112=E$2:E111)))))</f>
-        <v>SBJ_2</v>
-      </c>
-      <c r="J112" s="25">
+        <v/>
+      </c>
+      <c r="J112" s="25" t="str">
         <f ca="1">IF(OR(E112="",E112="!!!",F112="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E112)*(E112=E$2:E112)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E111)*(E2=E$1:E111))))))</f>
-        <v>0</v>
-      </c>
-      <c r="K112" s="25">
-        <f ca="1">IF(OR(E112="",E112="!!!",F112="NEW"),"",INDEX(J$1:J111,SUMPRODUCT(MAX(ROW(E$1:E111)*(E112=E$1:E111)))))</f>
-        <v>0</v>
-      </c>
-      <c r="L112" s="26"/>
+        <v/>
+      </c>
+      <c r="K112" s="25" t="str">
+        <f>IF(OR(E112="",E112="!!!",F112="NEW"),"",INDEX(J$1:J111,SUMPRODUCT(MAX(ROW(E$1:E111)*(E112=E$1:E111)))))</f>
+        <v/>
+      </c>
+      <c r="L112" s="26" t="s">
+        <v>483</v>
+      </c>
     </row>
     <row r="113" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
@@ -6212,10 +6165,10 @@
         <v>37</v>
       </c>
       <c r="E113" s="21" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="F113" s="22" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="G113" s="23" t="e">
         <f ca="1">IF(OR(E113="",E113="!!!"),"",IF(OR(J113=0,AND(J113=1,K113=1),AND(J113=1,I113="SBJ"),AND(J113=1,I113=0)),"?IN_FOCUS",IF(J113&lt;=2,"?ACTIVATED",IF(J113&lt;&gt;"","?FAMILIAR",IF(F113="NEW",IF(ISNA(VLOOKUP(E113,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
@@ -6238,7 +6191,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="L113" s="26" t="s">
-        <v>437</v>
+        <v>500</v>
       </c>
     </row>
     <row r="114" spans="1:12" x14ac:dyDescent="0.3">
@@ -6425,7 +6378,7 @@
         <v>37</v>
       </c>
       <c r="E119" s="21" t="s">
-        <v>440</v>
+        <v>434</v>
       </c>
       <c r="F119" s="22" t="str">
         <f>IF(OR(E119="",E119="!!!"),"",IF(NOT(ISNA(VLOOKUP(E119,E$1:E118,1,FALSE()))),"OLD",IF(AND(E119&lt;&gt;"",E119&lt;&gt;"!!!"),"NEW","")))</f>
@@ -6743,16 +6696,14 @@
       <c r="A128" t="s">
         <v>79</v>
       </c>
-      <c r="E128" s="21" t="s">
-        <v>422</v>
-      </c>
+      <c r="E128" s="21"/>
       <c r="F128" s="22" t="str">
         <f>IF(OR(E128="",E128="!!!"),"",IF(NOT(ISNA(VLOOKUP(E128,E$1:E127,1,FALSE()))),"OLD",IF(AND(E128&lt;&gt;"",E128&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v/>
       </c>
       <c r="G128" s="23" t="str">
-        <f ca="1">IF(OR(E128="",E128="!!!"),"",IF(OR(J128=0,AND(J128=1,K128=1),AND(J128=1,I128="SBJ"),AND(J128=1,I128=0)),"?IN_FOCUS",IF(J128&lt;=2,"?ACTIVATED",IF(J128&lt;&gt;"","?FAMILIAR",IF(F128="NEW",IF(ISNA(VLOOKUP(E128,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E128="",E128="!!!"),"",IF(OR(J128=0,AND(J128=1,K128=1),AND(J128=1,I128="SBJ"),AND(J128=1,I128=0)),"?IN_FOCUS",IF(J128&lt;=2,"?ACTIVATED",IF(J128&lt;&gt;"","?FAMILIAR",IF(F128="NEW",IF(ISNA(VLOOKUP(E128,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H128" s="24" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -6760,19 +6711,17 @@
       </c>
       <c r="I128" s="25" t="str">
         <f>IF(OR(E128="",E128="!!!",F128="NEW"),"",INDEX(B$2:B127,-1+SUMPRODUCT(MAX(ROW(E$2:E127)*(E128=E$2:E127)))))</f>
-        <v>other_2</v>
-      </c>
-      <c r="J128" s="25">
+        <v/>
+      </c>
+      <c r="J128" s="25" t="str">
         <f ca="1">IF(OR(E128="",E128="!!!",F128="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E128)*(E128=E$2:E128)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E127)*(E2=E$1:E127))))))</f>
-        <v>0</v>
-      </c>
-      <c r="K128" s="25">
-        <f ca="1">IF(OR(E128="",E128="!!!",F128="NEW"),"",INDEX(J$1:J127,SUMPRODUCT(MAX(ROW(E$1:E127)*(E128=E$1:E127)))))</f>
-        <v>0</v>
-      </c>
-      <c r="L128" s="26" t="s">
-        <v>425</v>
-      </c>
+        <v/>
+      </c>
+      <c r="K128" s="25" t="str">
+        <f>IF(OR(E128="",E128="!!!",F128="NEW"),"",INDEX(J$1:J127,SUMPRODUCT(MAX(ROW(E$1:E127)*(E128=E$1:E127)))))</f>
+        <v/>
+      </c>
+      <c r="L128" s="26"/>
     </row>
     <row r="129" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
@@ -6788,11 +6737,10 @@
         <v>37</v>
       </c>
       <c r="E129" s="21" t="s">
-        <v>441</v>
-      </c>
-      <c r="F129" s="22" t="str">
-        <f>IF(OR(E129="",E129="!!!"),"",IF(NOT(ISNA(VLOOKUP(E129,E$1:E128,1,FALSE()))),"OLD",IF(AND(E129&lt;&gt;"",E129&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>NEW</v>
+        <v>485</v>
+      </c>
+      <c r="F129" s="22" t="s">
+        <v>475</v>
       </c>
       <c r="G129" s="23" t="str">
         <f ca="1">IF(OR(E129="",E129="!!!"),"",IF(OR(J129=0,AND(J129=1,K129=1),AND(J129=1,I129="SBJ"),AND(J129=1,I129=0)),"?IN_FOCUS",IF(J129&lt;=2,"?ACTIVATED",IF(J129&lt;&gt;"","?FAMILIAR",IF(F129="NEW",IF(ISNA(VLOOKUP(E129,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
@@ -6814,7 +6762,9 @@
         <f>IF(OR(E129="",E129="!!!",F129="NEW"),"",INDEX(J$1:J128,SUMPRODUCT(MAX(ROW(E$1:E128)*(E129=E$1:E128)))))</f>
         <v/>
       </c>
-      <c r="L129" s="26"/>
+      <c r="L129" s="26" t="s">
+        <v>486</v>
+      </c>
     </row>
     <row r="130" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
@@ -6860,31 +6810,29 @@
       <c r="C131" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="E131" s="21" t="s">
-        <v>442</v>
-      </c>
+      <c r="E131" s="21"/>
       <c r="F131" s="22" t="str">
         <f>IF(OR(E131="",E131="!!!"),"",IF(NOT(ISNA(VLOOKUP(E131,E$1:E130,1,FALSE()))),"OLD",IF(AND(E131&lt;&gt;"",E131&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v/>
       </c>
       <c r="G131" s="23" t="str">
-        <f ca="1">IF(OR(E131="",E131="!!!"),"",IF(OR(J131=0,AND(J131=1,K131=1),AND(J131=1,I131="SBJ"),AND(J131=1,I131=0)),"?IN_FOCUS",IF(J131&lt;=2,"?ACTIVATED",IF(J131&lt;&gt;"","?FAMILIAR",IF(F131="NEW",IF(ISNA(VLOOKUP(E131,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E131="",E131="!!!"),"",IF(OR(J131=0,AND(J131=1,K131=1),AND(J131=1,I131="SBJ"),AND(J131=1,I131=0)),"?IN_FOCUS",IF(J131&lt;=2,"?ACTIVATED",IF(J131&lt;&gt;"","?FAMILIAR",IF(F131="NEW",IF(ISNA(VLOOKUP(E131,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H131" s="24" t="str">
         <f t="shared" ref="H131:H194" ca="1" si="4">IF(J131&lt;&gt;1,"",IF(I131="SBJ","CB","?"))</f>
         <v/>
       </c>
-      <c r="I131" s="25">
+      <c r="I131" s="25" t="str">
         <f>IF(OR(E131="",E131="!!!",F131="NEW"),"",INDEX(B$2:B130,-1+SUMPRODUCT(MAX(ROW(E$2:E130)*(E131=E$2:E130)))))</f>
-        <v>0</v>
-      </c>
-      <c r="J131" s="25">
+        <v/>
+      </c>
+      <c r="J131" s="25" t="str">
         <f ca="1">IF(OR(E131="",E131="!!!",F131="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E131)*(E131=E$2:E131)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E130)*(E2=E$1:E130))))))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K131" s="25" t="str">
-        <f ca="1">IF(OR(E131="",E131="!!!",F131="NEW"),"",INDEX(J$1:J130,SUMPRODUCT(MAX(ROW(E$1:E130)*(E131=E$1:E130)))))</f>
+        <f>IF(OR(E131="",E131="!!!",F131="NEW"),"",INDEX(J$1:J130,SUMPRODUCT(MAX(ROW(E$1:E130)*(E131=E$1:E130)))))</f>
         <v/>
       </c>
       <c r="L131" s="26"/>
@@ -6894,7 +6842,7 @@
         <v>130</v>
       </c>
       <c r="E132" s="21" t="str">
-        <f t="shared" ref="E131:E194" si="5">IF(D132="?OLD","!!!","")</f>
+        <f t="shared" ref="E132:E194" si="5">IF(D132="?OLD","!!!","")</f>
         <v/>
       </c>
       <c r="F132" s="22" t="str">
@@ -6967,16 +6915,14 @@
       <c r="C134" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="E134" s="21" t="s">
-        <v>458</v>
-      </c>
+      <c r="E134" s="21"/>
       <c r="F134" s="22" t="str">
         <f>IF(OR(E134="",E134="!!!"),"",IF(NOT(ISNA(VLOOKUP(E134,E$1:E133,1,FALSE()))),"OLD",IF(AND(E134&lt;&gt;"",E134&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>NEW</v>
+        <v/>
       </c>
       <c r="G134" s="23" t="str">
-        <f ca="1">IF(OR(E134="",E134="!!!"),"",IF(OR(J134=0,AND(J134=1,K134=1),AND(J134=1,I134="SBJ"),AND(J134=1,I134=0)),"?IN_FOCUS",IF(J134&lt;=2,"?ACTIVATED",IF(J134&lt;&gt;"","?FAMILIAR",IF(F134="NEW",IF(ISNA(VLOOKUP(E134,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?REFERENTIAL</v>
+        <f>IF(OR(E134="",E134="!!!"),"",IF(OR(J134=0,AND(J134=1,K134=1),AND(J134=1,I134="SBJ"),AND(J134=1,I134=0)),"?IN_FOCUS",IF(J134&lt;=2,"?ACTIVATED",IF(J134&lt;&gt;"","?FAMILIAR",IF(F134="NEW",IF(ISNA(VLOOKUP(E134,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H134" s="24" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -6994,9 +6940,7 @@
         <f>IF(OR(E134="",E134="!!!",F134="NEW"),"",INDEX(J$1:J133,SUMPRODUCT(MAX(ROW(E$1:E133)*(E134=E$1:E133)))))</f>
         <v/>
       </c>
-      <c r="L134" s="26" t="s">
-        <v>447</v>
-      </c>
+      <c r="L134" s="26"/>
     </row>
     <row r="135" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
@@ -7086,9 +7030,8 @@
         <v>37</v>
       </c>
       <c r="E137" s="21"/>
-      <c r="F137" s="22" t="str">
-        <f>IF(OR(E137="",E137="!!!"),"",IF(NOT(ISNA(VLOOKUP(E137,E$1:E136,1,FALSE()))),"OLD",IF(AND(E137&lt;&gt;"",E137&lt;&gt;"!!!"),"NEW","")))</f>
-        <v/>
+      <c r="F137" s="22" t="s">
+        <v>436</v>
       </c>
       <c r="G137" s="23" t="str">
         <f>IF(OR(E137="",E137="!!!"),"",IF(OR(J137=0,AND(J137=1,K137=1),AND(J137=1,I137="SBJ"),AND(J137=1,I137=0)),"?IN_FOCUS",IF(J137&lt;=2,"?ACTIVATED",IF(J137&lt;&gt;"","?FAMILIAR",IF(F137="NEW",IF(ISNA(VLOOKUP(E137,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
@@ -7110,9 +7053,7 @@
         <f>IF(OR(E137="",E137="!!!",F137="NEW"),"",INDEX(J$1:J136,SUMPRODUCT(MAX(ROW(E$1:E136)*(E137=E$1:E136)))))</f>
         <v/>
       </c>
-      <c r="L137" s="26" t="s">
-        <v>429</v>
-      </c>
+      <c r="L137" s="26"/>
     </row>
     <row r="138" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
@@ -7292,7 +7233,7 @@
       </c>
       <c r="L142" s="26"/>
     </row>
-    <row r="143" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>153</v>
       </c>
@@ -7303,10 +7244,10 @@
         <v>62</v>
       </c>
       <c r="E143" s="21" t="s">
-        <v>443</v>
+        <v>435</v>
       </c>
       <c r="F143" s="22" t="s">
-        <v>502</v>
+        <v>475</v>
       </c>
       <c r="G143" s="23" t="str">
         <f ca="1">IF(OR(E143="",E143="!!!"),"",IF(OR(J143=0,AND(J143=1,K143=1),AND(J143=1,I143="SBJ"),AND(J143=1,I143=0)),"?IN_FOCUS",IF(J143&lt;=2,"?ACTIVATED",IF(J143&lt;&gt;"","?FAMILIAR",IF(F143="NEW",IF(ISNA(VLOOKUP(E143,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
@@ -7329,7 +7270,7 @@
         <v/>
       </c>
       <c r="L143" s="26" t="s">
-        <v>501</v>
+        <v>484</v>
       </c>
     </row>
     <row r="144" spans="1:12" x14ac:dyDescent="0.3">
@@ -7373,16 +7314,14 @@
       <c r="B145" s="20" t="s">
         <v>155</v>
       </c>
-      <c r="E145" s="21" t="s">
-        <v>443</v>
-      </c>
+      <c r="E145" s="21"/>
       <c r="F145" s="22" t="str">
         <f>IF(OR(E145="",E145="!!!"),"",IF(NOT(ISNA(VLOOKUP(E145,E$1:E144,1,FALSE()))),"OLD",IF(AND(E145&lt;&gt;"",E145&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v/>
       </c>
       <c r="G145" s="23" t="str">
-        <f ca="1">IF(OR(E145="",E145="!!!"),"",IF(OR(J145=0,AND(J145=1,K145=1),AND(J145=1,I145="SBJ"),AND(J145=1,I145=0)),"?IN_FOCUS",IF(J145&lt;=2,"?ACTIVATED",IF(J145&lt;&gt;"","?FAMILIAR",IF(F145="NEW",IF(ISNA(VLOOKUP(E145,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E145="",E145="!!!"),"",IF(OR(J145=0,AND(J145=1,K145=1),AND(J145=1,I145="SBJ"),AND(J145=1,I145=0)),"?IN_FOCUS",IF(J145&lt;=2,"?ACTIVATED",IF(J145&lt;&gt;"","?FAMILIAR",IF(F145="NEW",IF(ISNA(VLOOKUP(E145,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H145" s="24" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -7390,14 +7329,14 @@
       </c>
       <c r="I145" s="25" t="str">
         <f>IF(OR(E145="",E145="!!!",F145="NEW"),"",INDEX(B$2:B144,-1+SUMPRODUCT(MAX(ROW(E$2:E144)*(E145=E$2:E144)))))</f>
-        <v>OBJ_3</v>
-      </c>
-      <c r="J145" s="25">
+        <v/>
+      </c>
+      <c r="J145" s="25" t="str">
         <f ca="1">IF(OR(E145="",E145="!!!",F145="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E145)*(E145=E$2:E145)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E144)*(E2=E$1:E144))))))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K145" s="25" t="str">
-        <f ca="1">IF(OR(E145="",E145="!!!",F145="NEW"),"",INDEX(J$1:J144,SUMPRODUCT(MAX(ROW(E$1:E144)*(E145=E$1:E144)))))</f>
+        <f>IF(OR(E145="",E145="!!!",F145="NEW"),"",INDEX(J$1:J144,SUMPRODUCT(MAX(ROW(E$1:E144)*(E145=E$1:E144)))))</f>
         <v/>
       </c>
       <c r="L145" s="26"/>
@@ -7625,7 +7564,7 @@
         <v>37</v>
       </c>
       <c r="E152" s="21" t="s">
-        <v>443</v>
+        <v>435</v>
       </c>
       <c r="F152" s="22" t="str">
         <f>IF(OR(E152="",E152="!!!"),"",IF(NOT(ISNA(VLOOKUP(E152,E$1:E151,1,FALSE()))),"OLD",IF(AND(E152&lt;&gt;"",E152&lt;&gt;"!!!"),"NEW","")))</f>
@@ -7641,15 +7580,15 @@
       </c>
       <c r="I152" s="25" t="str">
         <f>IF(OR(E152="",E152="!!!",F152="NEW"),"",INDEX(B$2:B151,-1+SUMPRODUCT(MAX(ROW(E$2:E151)*(E152=E$2:E151)))))</f>
-        <v>OBJ_5</v>
+        <v>OBJ_3</v>
       </c>
       <c r="J152" s="25">
         <f ca="1">IF(OR(E152="",E152="!!!",F152="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E152)*(E152=E$2:E152)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E151)*(E2=E$1:E151))))))</f>
         <v>0</v>
       </c>
-      <c r="K152" s="25">
+      <c r="K152" s="25" t="str">
         <f ca="1">IF(OR(E152="",E152="!!!",F152="NEW"),"",INDEX(J$1:J151,SUMPRODUCT(MAX(ROW(E$1:E151)*(E152=E$1:E151)))))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="L152" s="26"/>
     </row>
@@ -7763,10 +7702,10 @@
         <v/>
       </c>
       <c r="L155" s="26" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.3">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="156" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>162</v>
       </c>
@@ -7780,15 +7719,15 @@
         <v>37</v>
       </c>
       <c r="E156" s="21" t="s">
-        <v>445</v>
+        <v>485</v>
       </c>
       <c r="F156" s="22" t="str">
         <f>IF(OR(E156="",E156="!!!"),"",IF(NOT(ISNA(VLOOKUP(E156,E$1:E155,1,FALSE()))),"OLD",IF(AND(E156&lt;&gt;"",E156&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>NEW</v>
+        <v>OLD</v>
       </c>
       <c r="G156" s="23" t="str">
         <f ca="1">IF(OR(E156="",E156="!!!"),"",IF(OR(J156=0,AND(J156=1,K156=1),AND(J156=1,I156="SBJ"),AND(J156=1,I156=0)),"?IN_FOCUS",IF(J156&lt;=2,"?ACTIVATED",IF(J156&lt;&gt;"","?FAMILIAR",IF(F156="NEW",IF(ISNA(VLOOKUP(E156,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?REFERENTIAL</v>
+        <v>?IN_FOCUS</v>
       </c>
       <c r="H156" s="24" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -7796,17 +7735,19 @@
       </c>
       <c r="I156" s="25" t="str">
         <f>IF(OR(E156="",E156="!!!",F156="NEW"),"",INDEX(B$2:B155,-1+SUMPRODUCT(MAX(ROW(E$2:E155)*(E156=E$2:E155)))))</f>
-        <v/>
-      </c>
-      <c r="J156" s="25" t="str">
+        <v>other</v>
+      </c>
+      <c r="J156" s="25">
         <f ca="1">IF(OR(E156="",E156="!!!",F156="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E156)*(E156=E$2:E156)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E155)*(E2=E$1:E155))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K156" s="25" t="str">
-        <f>IF(OR(E156="",E156="!!!",F156="NEW"),"",INDEX(J$1:J155,SUMPRODUCT(MAX(ROW(E$1:E155)*(E156=E$1:E155)))))</f>
-        <v/>
-      </c>
-      <c r="L156" s="26"/>
+        <f ca="1">IF(OR(E156="",E156="!!!",F156="NEW"),"",INDEX(J$1:J155,SUMPRODUCT(MAX(ROW(E$1:E155)*(E156=E$1:E155)))))</f>
+        <v/>
+      </c>
+      <c r="L156" s="26" t="s">
+        <v>487</v>
+      </c>
     </row>
     <row r="157" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
@@ -8278,7 +8219,7 @@
         <v>37</v>
       </c>
       <c r="E170" s="21" t="s">
-        <v>456</v>
+        <v>445</v>
       </c>
       <c r="F170" s="22" t="str">
         <f>IF(OR(E170="",E170="!!!"),"",IF(NOT(ISNA(VLOOKUP(E170,E$1:E169,1,FALSE()))),"OLD",IF(AND(E170&lt;&gt;"",E170&lt;&gt;"!!!"),"NEW","")))</f>
@@ -8305,7 +8246,7 @@
         <v/>
       </c>
       <c r="L170" s="26" t="s">
-        <v>457</v>
+        <v>446</v>
       </c>
     </row>
     <row r="171" spans="1:12" x14ac:dyDescent="0.3">
@@ -8356,7 +8297,7 @@
         <v>37</v>
       </c>
       <c r="E172" s="21" t="s">
-        <v>446</v>
+        <v>437</v>
       </c>
       <c r="F172" s="22" t="str">
         <f>IF(OR(E172="",E172="!!!"),"",IF(NOT(ISNA(VLOOKUP(E172,E$1:E171,1,FALSE()))),"OLD",IF(AND(E172&lt;&gt;"",E172&lt;&gt;"!!!"),"NEW","")))</f>
@@ -8457,7 +8398,7 @@
         <v/>
       </c>
       <c r="L174" s="26" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
     </row>
     <row r="175" spans="1:12" x14ac:dyDescent="0.3">
@@ -8488,9 +8429,9 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-      <c r="I175" s="25">
+      <c r="I175" s="25" t="str">
         <f>IF(OR(E175="",E175="!!!",F175="NEW"),"",INDEX(B$2:B174,-1+SUMPRODUCT(MAX(ROW(E$2:E174)*(E175=E$2:E174)))))</f>
-        <v>0</v>
+        <v>other_2</v>
       </c>
       <c r="J175" s="25">
         <f ca="1">IF(OR(E175="",E175="!!!",F175="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E175)*(E175=E$2:E175)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E174)*(E2=E$1:E174))))))</f>
@@ -8541,7 +8482,7 @@
         <v>174</v>
       </c>
       <c r="E177" s="21" t="s">
-        <v>456</v>
+        <v>445</v>
       </c>
       <c r="F177" s="22" t="str">
         <f>IF(OR(E177="",E177="!!!"),"",IF(NOT(ISNA(VLOOKUP(E177,E$1:E176,1,FALSE()))),"OLD",IF(AND(E177&lt;&gt;"",E177&lt;&gt;"!!!"),"NEW","")))</f>
@@ -8580,10 +8521,10 @@
         <v>176</v>
       </c>
       <c r="E178" s="21" t="s">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="F178" s="22" t="s">
-        <v>444</v>
+        <v>436</v>
       </c>
       <c r="G178" s="23" t="e">
         <f ca="1">IF(OR(E178="",E178="!!!"),"",IF(OR(J178=0,AND(J178=1,K178=1),AND(J178=1,I178="SBJ"),AND(J178=1,I178=0)),"?IN_FOCUS",IF(J178&lt;=2,"?ACTIVATED",IF(J178&lt;&gt;"","?FAMILIAR",IF(F178="NEW",IF(ISNA(VLOOKUP(E178,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
@@ -8606,7 +8547,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="L178" s="26" t="s">
-        <v>493</v>
+        <v>470</v>
       </c>
     </row>
     <row r="179" spans="1:12" x14ac:dyDescent="0.3">
@@ -8725,33 +8666,33 @@
         <v>37</v>
       </c>
       <c r="E182" s="21" t="s">
-        <v>460</v>
+        <v>448</v>
       </c>
       <c r="F182" s="22" t="s">
-        <v>485</v>
-      </c>
-      <c r="G182" s="23" t="e">
+        <v>475</v>
+      </c>
+      <c r="G182" s="23" t="str">
         <f ca="1">IF(OR(E182="",E182="!!!"),"",IF(OR(J182=0,AND(J182=1,K182=1),AND(J182=1,I182="SBJ"),AND(J182=1,I182=0)),"?IN_FOCUS",IF(J182&lt;=2,"?ACTIVATED",IF(J182&lt;&gt;"","?FAMILIAR",IF(F182="NEW",IF(ISNA(VLOOKUP(E182,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>#VALUE!</v>
+        <v>?REFERENTIAL</v>
       </c>
       <c r="H182" s="24" t="str">
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-      <c r="I182" s="25" t="e">
+      <c r="I182" s="25" t="str">
         <f>IF(OR(E182="",E182="!!!",F182="NEW"),"",INDEX(B$2:B181,-1+SUMPRODUCT(MAX(ROW(E$2:E181)*(E182=E$2:E181)))))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="J182" s="25">
+        <v/>
+      </c>
+      <c r="J182" s="25" t="str">
         <f ca="1">IF(OR(E182="",E182="!!!",F182="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E182)*(E182=E$2:E182)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E181)*(E2=E$1:E181))))))</f>
-        <v>0</v>
-      </c>
-      <c r="K182" s="25" t="e">
+        <v/>
+      </c>
+      <c r="K182" s="25" t="str">
         <f>IF(OR(E182="",E182="!!!",F182="NEW"),"",INDEX(J$1:J181,SUMPRODUCT(MAX(ROW(E$1:E181)*(E182=E$1:E181)))))</f>
-        <v>#VALUE!</v>
+        <v/>
       </c>
       <c r="L182" s="26" t="s">
-        <v>503</v>
+        <v>488</v>
       </c>
     </row>
     <row r="183" spans="1:12" x14ac:dyDescent="0.3">
@@ -9047,16 +8988,13 @@
       <c r="D191" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="E191" s="21" t="s">
-        <v>460</v>
-      </c>
-      <c r="F191" s="22" t="str">
-        <f>IF(OR(E191="",E191="!!!"),"",IF(NOT(ISNA(VLOOKUP(E191,E$1:E190,1,FALSE()))),"OLD",IF(AND(E191&lt;&gt;"",E191&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+      <c r="E191" s="21"/>
+      <c r="F191" s="22" t="s">
+        <v>444</v>
       </c>
       <c r="G191" s="23" t="str">
-        <f ca="1">IF(OR(E191="",E191="!!!"),"",IF(OR(J191=0,AND(J191=1,K191=1),AND(J191=1,I191="SBJ"),AND(J191=1,I191=0)),"?IN_FOCUS",IF(J191&lt;=2,"?ACTIVATED",IF(J191&lt;&gt;"","?FAMILIAR",IF(F191="NEW",IF(ISNA(VLOOKUP(E191,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E191="",E191="!!!"),"",IF(OR(J191=0,AND(J191=1,K191=1),AND(J191=1,I191="SBJ"),AND(J191=1,I191=0)),"?IN_FOCUS",IF(J191&lt;=2,"?ACTIVATED",IF(J191&lt;&gt;"","?FAMILIAR",IF(F191="NEW",IF(ISNA(VLOOKUP(E191,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H191" s="24" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -9064,15 +9002,15 @@
       </c>
       <c r="I191" s="25" t="str">
         <f>IF(OR(E191="",E191="!!!",F191="NEW"),"",INDEX(B$2:B190,-1+SUMPRODUCT(MAX(ROW(E$2:E190)*(E191=E$2:E190)))))</f>
-        <v>SBJ_4</v>
-      </c>
-      <c r="J191" s="25">
+        <v/>
+      </c>
+      <c r="J191" s="25" t="str">
         <f ca="1">IF(OR(E191="",E191="!!!",F191="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E191)*(E191=E$2:E191)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E190)*(E2=E$1:E190))))))</f>
-        <v>0</v>
-      </c>
-      <c r="K191" s="25">
-        <f ca="1">IF(OR(E191="",E191="!!!",F191="NEW"),"",INDEX(J$1:J190,SUMPRODUCT(MAX(ROW(E$1:E190)*(E191=E$1:E190)))))</f>
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="K191" s="25" t="str">
+        <f>IF(OR(E191="",E191="!!!",F191="NEW"),"",INDEX(J$1:J190,SUMPRODUCT(MAX(ROW(E$1:E190)*(E191=E$1:E190)))))</f>
+        <v/>
       </c>
       <c r="L191" s="26"/>
     </row>
@@ -9117,16 +9055,14 @@
       <c r="B193" s="20" t="s">
         <v>156</v>
       </c>
-      <c r="E193" s="21" t="s">
-        <v>460</v>
-      </c>
+      <c r="E193" s="21"/>
       <c r="F193" s="22" t="str">
         <f>IF(OR(E193="",E193="!!!"),"",IF(NOT(ISNA(VLOOKUP(E193,E$1:E192,1,FALSE()))),"OLD",IF(AND(E193&lt;&gt;"",E193&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v/>
       </c>
       <c r="G193" s="23" t="str">
-        <f ca="1">IF(OR(E193="",E193="!!!"),"",IF(OR(J193=0,AND(J193=1,K193=1),AND(J193=1,I193="SBJ"),AND(J193=1,I193=0)),"?IN_FOCUS",IF(J193&lt;=2,"?ACTIVATED",IF(J193&lt;&gt;"","?FAMILIAR",IF(F193="NEW",IF(ISNA(VLOOKUP(E193,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E193="",E193="!!!"),"",IF(OR(J193=0,AND(J193=1,K193=1),AND(J193=1,I193="SBJ"),AND(J193=1,I193=0)),"?IN_FOCUS",IF(J193&lt;=2,"?ACTIVATED",IF(J193&lt;&gt;"","?FAMILIAR",IF(F193="NEW",IF(ISNA(VLOOKUP(E193,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H193" s="24" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -9134,15 +9070,15 @@
       </c>
       <c r="I193" s="25" t="str">
         <f>IF(OR(E193="",E193="!!!",F193="NEW"),"",INDEX(B$2:B192,-1+SUMPRODUCT(MAX(ROW(E$2:E192)*(E193=E$2:E192)))))</f>
-        <v>SBJ_3</v>
-      </c>
-      <c r="J193" s="25">
+        <v/>
+      </c>
+      <c r="J193" s="25" t="str">
         <f ca="1">IF(OR(E193="",E193="!!!",F193="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E193)*(E193=E$2:E193)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E192)*(E2=E$1:E192))))))</f>
-        <v>0</v>
-      </c>
-      <c r="K193" s="25">
-        <f ca="1">IF(OR(E193="",E193="!!!",F193="NEW"),"",INDEX(J$1:J192,SUMPRODUCT(MAX(ROW(E$1:E192)*(E193=E$1:E192)))))</f>
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="K193" s="25" t="str">
+        <f>IF(OR(E193="",E193="!!!",F193="NEW"),"",INDEX(J$1:J192,SUMPRODUCT(MAX(ROW(E$1:E192)*(E193=E$1:E192)))))</f>
+        <v/>
       </c>
       <c r="L193" s="26"/>
     </row>
@@ -9302,7 +9238,7 @@
         <v>37</v>
       </c>
       <c r="E198" s="21" t="s">
-        <v>460</v>
+        <v>448</v>
       </c>
       <c r="F198" s="22" t="str">
         <f>IF(OR(E198="",E198="!!!"),"",IF(NOT(ISNA(VLOOKUP(E198,E$1:E197,1,FALSE()))),"OLD",IF(AND(E198&lt;&gt;"",E198&lt;&gt;"!!!"),"NEW","")))</f>
@@ -9318,15 +9254,15 @@
       </c>
       <c r="I198" s="25" t="str">
         <f>IF(OR(E198="",E198="!!!",F198="NEW"),"",INDEX(B$2:B197,-1+SUMPRODUCT(MAX(ROW(E$2:E197)*(E198=E$2:E197)))))</f>
-        <v>SBJ_5</v>
+        <v>SBJ_4</v>
       </c>
       <c r="J198" s="25">
         <f ca="1">IF(OR(E198="",E198="!!!",F198="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E198)*(E198=E$2:E198)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E197)*(E2=E$1:E197))))))</f>
         <v>0</v>
       </c>
-      <c r="K198" s="25">
+      <c r="K198" s="25" t="str">
         <f ca="1">IF(OR(E198="",E198="!!!",F198="NEW"),"",INDEX(J$1:J197,SUMPRODUCT(MAX(ROW(E$1:E197)*(E198=E$1:E197)))))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="L198" s="26"/>
     </row>
@@ -9514,10 +9450,10 @@
         <v>37</v>
       </c>
       <c r="E204" s="21" t="s">
-        <v>448</v>
+        <v>439</v>
       </c>
       <c r="F204" s="22" t="s">
-        <v>444</v>
+        <v>436</v>
       </c>
       <c r="G204" s="23" t="e">
         <f ca="1">IF(OR(E204="",E204="!!!"),"",IF(OR(J204=0,AND(J204=1,K204=1),AND(J204=1,I204="SBJ"),AND(J204=1,I204=0)),"?IN_FOCUS",IF(J204&lt;=2,"?ACTIVATED",IF(J204&lt;&gt;"","?FAMILIAR",IF(F204="NEW",IF(ISNA(VLOOKUP(E204,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
@@ -9540,7 +9476,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="L204" s="26" t="s">
-        <v>478</v>
+        <v>465</v>
       </c>
     </row>
     <row r="205" spans="1:12" x14ac:dyDescent="0.3">
@@ -9624,31 +9560,29 @@
       <c r="D207" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="E207" s="21" t="s">
-        <v>454</v>
-      </c>
+      <c r="E207" s="21"/>
       <c r="F207" s="22" t="s">
-        <v>455</v>
-      </c>
-      <c r="G207" s="23" t="e">
-        <f ca="1">IF(OR(E207="",E207="!!!"),"",IF(OR(J207=0,AND(J207=1,K207=1),AND(J207=1,I207="SBJ"),AND(J207=1,I207=0)),"?IN_FOCUS",IF(J207&lt;=2,"?ACTIVATED",IF(J207&lt;&gt;"","?FAMILIAR",IF(F207="NEW",IF(ISNA(VLOOKUP(E207,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>#VALUE!</v>
+        <v>444</v>
+      </c>
+      <c r="G207" s="23" t="str">
+        <f>IF(OR(E207="",E207="!!!"),"",IF(OR(J207=0,AND(J207=1,K207=1),AND(J207=1,I207="SBJ"),AND(J207=1,I207=0)),"?IN_FOCUS",IF(J207&lt;=2,"?ACTIVATED",IF(J207&lt;&gt;"","?FAMILIAR",IF(F207="NEW",IF(ISNA(VLOOKUP(E207,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H207" s="24" t="str">
         <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
-      <c r="I207" s="25" t="e">
+      <c r="I207" s="25" t="str">
         <f>IF(OR(E207="",E207="!!!",F207="NEW"),"",INDEX(B$2:B206,-1+SUMPRODUCT(MAX(ROW(E$2:E206)*(E207=E$2:E206)))))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="J207" s="25">
+        <v/>
+      </c>
+      <c r="J207" s="25" t="str">
         <f ca="1">IF(OR(E207="",E207="!!!",F207="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E207)*(E207=E$2:E207)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E206)*(E2=E$1:E206))))))</f>
-        <v>0</v>
-      </c>
-      <c r="K207" s="25" t="e">
+        <v/>
+      </c>
+      <c r="K207" s="25" t="str">
         <f>IF(OR(E207="",E207="!!!",F207="NEW"),"",INDEX(J$1:J206,SUMPRODUCT(MAX(ROW(E$1:E206)*(E207=E$1:E206)))))</f>
-        <v>#VALUE!</v>
+        <v/>
       </c>
       <c r="L207" s="26"/>
     </row>
@@ -9730,16 +9664,14 @@
       <c r="C210" s="20" t="s">
         <v>192</v>
       </c>
-      <c r="E210" s="21" t="s">
-        <v>454</v>
-      </c>
+      <c r="E210" s="21"/>
       <c r="F210" s="22" t="str">
         <f>IF(OR(E210="",E210="!!!"),"",IF(NOT(ISNA(VLOOKUP(E210,E$1:E209,1,FALSE()))),"OLD",IF(AND(E210&lt;&gt;"",E210&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v/>
       </c>
       <c r="G210" s="23" t="str">
-        <f ca="1">IF(OR(E210="",E210="!!!"),"",IF(OR(J210=0,AND(J210=1,K210=1),AND(J210=1,I210="SBJ"),AND(J210=1,I210=0)),"?IN_FOCUS",IF(J210&lt;=2,"?ACTIVATED",IF(J210&lt;&gt;"","?FAMILIAR",IF(F210="NEW",IF(ISNA(VLOOKUP(E210,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E210="",E210="!!!"),"",IF(OR(J210=0,AND(J210=1,K210=1),AND(J210=1,I210="SBJ"),AND(J210=1,I210=0)),"?IN_FOCUS",IF(J210&lt;=2,"?ACTIVATED",IF(J210&lt;&gt;"","?FAMILIAR",IF(F210="NEW",IF(ISNA(VLOOKUP(E210,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H210" s="24" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -9747,15 +9679,15 @@
       </c>
       <c r="I210" s="25" t="str">
         <f>IF(OR(E210="",E210="!!!",F210="NEW"),"",INDEX(B$2:B209,-1+SUMPRODUCT(MAX(ROW(E$2:E209)*(E210=E$2:E209)))))</f>
-        <v>OBJ_3</v>
-      </c>
-      <c r="J210" s="25">
+        <v/>
+      </c>
+      <c r="J210" s="25" t="str">
         <f ca="1">IF(OR(E210="",E210="!!!",F210="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E210)*(E210=E$2:E210)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E209)*(E2=E$1:E209))))))</f>
-        <v>0</v>
-      </c>
-      <c r="K210" s="25">
-        <f ca="1">IF(OR(E210="",E210="!!!",F210="NEW"),"",INDEX(J$1:J209,SUMPRODUCT(MAX(ROW(E$1:E209)*(E210=E$1:E209)))))</f>
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="K210" s="25" t="str">
+        <f>IF(OR(E210="",E210="!!!",F210="NEW"),"",INDEX(J$1:J209,SUMPRODUCT(MAX(ROW(E$1:E209)*(E210=E$1:E209)))))</f>
+        <v/>
       </c>
       <c r="L210" s="26"/>
     </row>
@@ -9807,7 +9739,7 @@
         <v>37</v>
       </c>
       <c r="E212" s="21" t="s">
-        <v>446</v>
+        <v>437</v>
       </c>
       <c r="F212" s="22" t="str">
         <f>IF(OR(E212="",E212="!!!"),"",IF(NOT(ISNA(VLOOKUP(E212,E$1:E211,1,FALSE()))),"OLD",IF(AND(E212&lt;&gt;"",E212&lt;&gt;"!!!"),"NEW","")))</f>
@@ -9840,7 +9772,7 @@
         <v>194</v>
       </c>
       <c r="E213" s="21" t="s">
-        <v>446</v>
+        <v>437</v>
       </c>
       <c r="F213" s="22" t="str">
         <f>IF(OR(E213="",E213="!!!"),"",IF(NOT(ISNA(VLOOKUP(E213,E$1:E212,1,FALSE()))),"OLD",IF(AND(E213&lt;&gt;"",E213&lt;&gt;"!!!"),"NEW","")))</f>
@@ -9878,16 +9810,14 @@
       <c r="C214" s="20" t="s">
         <v>176</v>
       </c>
-      <c r="E214" s="21" t="s">
-        <v>449</v>
-      </c>
+      <c r="E214" s="21"/>
       <c r="F214" s="22" t="str">
         <f>IF(OR(E214="",E214="!!!"),"",IF(NOT(ISNA(VLOOKUP(E214,E$1:E213,1,FALSE()))),"OLD",IF(AND(E214&lt;&gt;"",E214&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>NEW</v>
+        <v/>
       </c>
       <c r="G214" s="23" t="str">
-        <f ca="1">IF(OR(E214="",E214="!!!"),"",IF(OR(J214=0,AND(J214=1,K214=1),AND(J214=1,I214="SBJ"),AND(J214=1,I214=0)),"?IN_FOCUS",IF(J214&lt;=2,"?ACTIVATED",IF(J214&lt;&gt;"","?FAMILIAR",IF(F214="NEW",IF(ISNA(VLOOKUP(E214,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?REFERENTIAL</v>
+        <f>IF(OR(E214="",E214="!!!"),"",IF(OR(J214=0,AND(J214=1,K214=1),AND(J214=1,I214="SBJ"),AND(J214=1,I214=0)),"?IN_FOCUS",IF(J214&lt;=2,"?ACTIVATED",IF(J214&lt;&gt;"","?FAMILIAR",IF(F214="NEW",IF(ISNA(VLOOKUP(E214,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H214" s="24" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -9905,9 +9835,7 @@
         <f>IF(OR(E214="",E214="!!!",F214="NEW"),"",INDEX(J$1:J213,SUMPRODUCT(MAX(ROW(E$1:E213)*(E214=E$1:E213)))))</f>
         <v/>
       </c>
-      <c r="L214" s="26" t="s">
-        <v>428</v>
-      </c>
+      <c r="L214" s="26"/>
     </row>
     <row r="215" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
@@ -9984,16 +9912,14 @@
       <c r="B217" s="20" t="s">
         <v>156</v>
       </c>
-      <c r="E217" s="21" t="s">
-        <v>449</v>
-      </c>
+      <c r="E217" s="21"/>
       <c r="F217" s="22" t="str">
         <f>IF(OR(E217="",E217="!!!"),"",IF(NOT(ISNA(VLOOKUP(E217,E$1:E216,1,FALSE()))),"OLD",IF(AND(E217&lt;&gt;"",E217&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v/>
       </c>
       <c r="G217" s="23" t="str">
-        <f ca="1">IF(OR(E217="",E217="!!!"),"",IF(OR(J217=0,AND(J217=1,K217=1),AND(J217=1,I217="SBJ"),AND(J217=1,I217=0)),"?IN_FOCUS",IF(J217&lt;=2,"?ACTIVATED",IF(J217&lt;&gt;"","?FAMILIAR",IF(F217="NEW",IF(ISNA(VLOOKUP(E217,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E217="",E217="!!!"),"",IF(OR(J217=0,AND(J217=1,K217=1),AND(J217=1,I217="SBJ"),AND(J217=1,I217=0)),"?IN_FOCUS",IF(J217&lt;=2,"?ACTIVATED",IF(J217&lt;&gt;"","?FAMILIAR",IF(F217="NEW",IF(ISNA(VLOOKUP(E217,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H217" s="24" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -10001,14 +9927,14 @@
       </c>
       <c r="I217" s="25" t="str">
         <f>IF(OR(E217="",E217="!!!",F217="NEW"),"",INDEX(B$2:B216,-1+SUMPRODUCT(MAX(ROW(E$2:E216)*(E217=E$2:E216)))))</f>
-        <v>OBJ_5</v>
-      </c>
-      <c r="J217" s="25">
+        <v/>
+      </c>
+      <c r="J217" s="25" t="str">
         <f ca="1">IF(OR(E217="",E217="!!!",F217="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E217)*(E217=E$2:E217)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E216)*(E2=E$1:E216))))))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K217" s="25" t="str">
-        <f ca="1">IF(OR(E217="",E217="!!!",F217="NEW"),"",INDEX(J$1:J216,SUMPRODUCT(MAX(ROW(E$1:E216)*(E217=E$1:E216)))))</f>
+        <f>IF(OR(E217="",E217="!!!",F217="NEW"),"",INDEX(J$1:J216,SUMPRODUCT(MAX(ROW(E$1:E216)*(E217=E$1:E216)))))</f>
         <v/>
       </c>
       <c r="L217" s="26"/>
@@ -10129,7 +10055,7 @@
         <v>37</v>
       </c>
       <c r="E221" s="21" t="s">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="F221" s="22" t="str">
         <f>IF(OR(E221="",E221="!!!"),"",IF(NOT(ISNA(VLOOKUP(E221,E$1:E220,1,FALSE()))),"OLD",IF(AND(E221&lt;&gt;"",E221&lt;&gt;"!!!"),"NEW","")))</f>
@@ -10375,7 +10301,7 @@
         <v>37</v>
       </c>
       <c r="E228" s="21" t="s">
-        <v>451</v>
+        <v>441</v>
       </c>
       <c r="F228" s="22" t="str">
         <f>IF(OR(E228="",E228="!!!"),"",IF(NOT(ISNA(VLOOKUP(E228,E$1:E227,1,FALSE()))),"OLD",IF(AND(E228&lt;&gt;"",E228&lt;&gt;"!!!"),"NEW","")))</f>
@@ -10452,7 +10378,7 @@
       </c>
       <c r="E230" s="21"/>
       <c r="F230" s="22" t="s">
-        <v>452</v>
+        <v>442</v>
       </c>
       <c r="G230" s="23" t="str">
         <f>IF(OR(E230="",E230="!!!"),"",IF(OR(J230=0,AND(J230=1,K230=1),AND(J230=1,I230="SBJ"),AND(J230=1,I230=0)),"?IN_FOCUS",IF(J230&lt;=2,"?ACTIVATED",IF(J230&lt;&gt;"","?FAMILIAR",IF(F230="NEW",IF(ISNA(VLOOKUP(E230,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
@@ -10475,7 +10401,7 @@
         <v/>
       </c>
       <c r="L230" s="26" t="s">
-        <v>453</v>
+        <v>443</v>
       </c>
     </row>
     <row r="231" spans="1:12" x14ac:dyDescent="0.3">
@@ -10850,7 +10776,7 @@
         <v>54</v>
       </c>
       <c r="E241" s="21" t="s">
-        <v>461</v>
+        <v>449</v>
       </c>
       <c r="F241" s="22" t="str">
         <f>IF(OR(E241="",E241="!!!"),"",IF(NOT(ISNA(VLOOKUP(E241,E$1:E240,1,FALSE()))),"OLD",IF(AND(E241&lt;&gt;"",E241&lt;&gt;"!!!"),"NEW","")))</f>
@@ -10877,7 +10803,7 @@
         <v/>
       </c>
       <c r="L241" s="26" t="s">
-        <v>462</v>
+        <v>450</v>
       </c>
     </row>
     <row r="242" spans="1:12" x14ac:dyDescent="0.3">
@@ -10962,7 +10888,7 @@
         <v>37</v>
       </c>
       <c r="E244" s="21" t="s">
-        <v>448</v>
+        <v>439</v>
       </c>
       <c r="F244" s="22" t="str">
         <f>IF(OR(E244="",E244="!!!"),"",IF(NOT(ISNA(VLOOKUP(E244,E$1:E243,1,FALSE()))),"OLD",IF(AND(E244&lt;&gt;"",E244&lt;&gt;"!!!"),"NEW","")))</f>
@@ -11171,7 +11097,7 @@
         <v>62</v>
       </c>
       <c r="E250" s="21" t="s">
-        <v>459</v>
+        <v>447</v>
       </c>
       <c r="F250" s="22" t="str">
         <f>IF(OR(E250="",E250="!!!"),"",IF(NOT(ISNA(VLOOKUP(E250,E$1:E249,1,FALSE()))),"OLD",IF(AND(E250&lt;&gt;"",E250&lt;&gt;"!!!"),"NEW","")))</f>
@@ -11664,7 +11590,7 @@
         <v/>
       </c>
       <c r="L263" s="26" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
     </row>
     <row r="264" spans="1:12" x14ac:dyDescent="0.3">
@@ -11701,12 +11627,12 @@
       </c>
       <c r="L264" s="26"/>
     </row>
-    <row r="265" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>184</v>
       </c>
       <c r="E265" s="21" t="s">
-        <v>460</v>
+        <v>448</v>
       </c>
       <c r="F265" s="22" t="str">
         <f>IF(OR(E265="",E265="!!!"),"",IF(NOT(ISNA(VLOOKUP(E265,E$1:E264,1,FALSE()))),"OLD",IF(AND(E265&lt;&gt;"",E265&lt;&gt;"!!!"),"NEW","")))</f>
@@ -11733,7 +11659,7 @@
         <v>0</v>
       </c>
       <c r="L265" s="26" t="s">
-        <v>504</v>
+        <v>489</v>
       </c>
     </row>
     <row r="266" spans="1:12" x14ac:dyDescent="0.3">
@@ -11855,7 +11781,7 @@
         <v>93</v>
       </c>
       <c r="E269" s="21" t="s">
-        <v>460</v>
+        <v>448</v>
       </c>
       <c r="F269" s="22" t="str">
         <f>IF(OR(E269="",E269="!!!"),"",IF(NOT(ISNA(VLOOKUP(E269,E$1:E268,1,FALSE()))),"OLD",IF(AND(E269&lt;&gt;"",E269&lt;&gt;"!!!"),"NEW","")))</f>
@@ -11995,16 +11921,14 @@
       <c r="C273" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="E273" s="21" t="s">
-        <v>476</v>
-      </c>
+      <c r="E273" s="21"/>
       <c r="F273" s="22" t="str">
         <f>IF(OR(E273="",E273="!!!"),"",IF(NOT(ISNA(VLOOKUP(E273,E$1:E272,1,FALSE()))),"OLD",IF(AND(E273&lt;&gt;"",E273&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>NEW</v>
+        <v/>
       </c>
       <c r="G273" s="23" t="str">
-        <f ca="1">IF(OR(E273="",E273="!!!"),"",IF(OR(J273=0,AND(J273=1,K273=1),AND(J273=1,I273="SBJ"),AND(J273=1,I273=0)),"?IN_FOCUS",IF(J273&lt;=2,"?ACTIVATED",IF(J273&lt;&gt;"","?FAMILIAR",IF(F273="NEW",IF(ISNA(VLOOKUP(E273,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?REFERENTIAL</v>
+        <f>IF(OR(E273="",E273="!!!"),"",IF(OR(J273=0,AND(J273=1,K273=1),AND(J273=1,I273="SBJ"),AND(J273=1,I273=0)),"?IN_FOCUS",IF(J273&lt;=2,"?ACTIVATED",IF(J273&lt;&gt;"","?FAMILIAR",IF(F273="NEW",IF(ISNA(VLOOKUP(E273,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H273" s="24" t="str">
         <f t="shared" ca="1" si="9"/>
@@ -12106,7 +12030,7 @@
         <v>37</v>
       </c>
       <c r="E276" s="21" t="s">
-        <v>474</v>
+        <v>502</v>
       </c>
       <c r="F276" s="22" t="str">
         <f>IF(OR(E276="",E276="!!!"),"",IF(NOT(ISNA(VLOOKUP(E276,E$1:E275,1,FALSE()))),"OLD",IF(AND(E276&lt;&gt;"",E276&lt;&gt;"!!!"),"NEW","")))</f>
@@ -12182,7 +12106,7 @@
         <v>37</v>
       </c>
       <c r="E278" s="21" t="s">
-        <v>461</v>
+        <v>449</v>
       </c>
       <c r="F278" s="22" t="str">
         <f>IF(OR(E278="",E278="!!!"),"",IF(NOT(ISNA(VLOOKUP(E278,E$1:E277,1,FALSE()))),"OLD",IF(AND(E278&lt;&gt;"",E278&lt;&gt;"!!!"),"NEW","")))</f>
@@ -12675,7 +12599,7 @@
         <v>37</v>
       </c>
       <c r="E292" s="21" t="s">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="F292" s="22" t="str">
         <f>IF(OR(E292="",E292="!!!"),"",IF(NOT(ISNA(VLOOKUP(E292,E$1:E291,1,FALSE()))),"OLD",IF(AND(E292&lt;&gt;"",E292&lt;&gt;"!!!"),"NEW","")))</f>
@@ -12701,7 +12625,9 @@
         <f ca="1">IF(OR(E292="",E292="!!!",F292="NEW"),"",INDEX(J$1:J291,SUMPRODUCT(MAX(ROW(E$1:E291)*(E292=E$1:E291)))))</f>
         <v>0</v>
       </c>
-      <c r="L292" s="26"/>
+      <c r="L292" s="26" t="s">
+        <v>490</v>
+      </c>
     </row>
     <row r="293" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
@@ -12853,7 +12779,7 @@
         <v>37</v>
       </c>
       <c r="E297" s="21" t="s">
-        <v>448</v>
+        <v>439</v>
       </c>
       <c r="F297" s="22" t="str">
         <f>IF(OR(E297="",E297="!!!"),"",IF(NOT(ISNA(VLOOKUP(E297,E$1:E296,1,FALSE()))),"OLD",IF(AND(E297&lt;&gt;"",E297&lt;&gt;"!!!"),"NEW","")))</f>
@@ -13032,7 +12958,7 @@
       </c>
       <c r="E302" s="21"/>
       <c r="F302" s="22" t="s">
-        <v>444</v>
+        <v>436</v>
       </c>
       <c r="G302" s="23" t="str">
         <f>IF(OR(E302="",E302="!!!"),"",IF(OR(J302=0,AND(J302=1,K302=1),AND(J302=1,I302="SBJ"),AND(J302=1,I302=0)),"?IN_FOCUS",IF(J302&lt;=2,"?ACTIVATED",IF(J302&lt;&gt;"","?FAMILIAR",IF(F302="NEW",IF(ISNA(VLOOKUP(E302,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
@@ -13055,7 +12981,7 @@
         <v/>
       </c>
       <c r="L302" s="26" t="s">
-        <v>463</v>
+        <v>451</v>
       </c>
     </row>
     <row r="303" spans="1:12" x14ac:dyDescent="0.3">
@@ -13106,7 +13032,7 @@
         <v>37</v>
       </c>
       <c r="E304" s="21" t="s">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="F304" s="22" t="str">
         <f>IF(OR(E304="",E304="!!!"),"",IF(NOT(ISNA(VLOOKUP(E304,E$1:E303,1,FALSE()))),"OLD",IF(AND(E304&lt;&gt;"",E304&lt;&gt;"!!!"),"NEW","")))</f>
@@ -13173,7 +13099,7 @@
         <v>249</v>
       </c>
       <c r="E306" s="21" t="s">
-        <v>464</v>
+        <v>452</v>
       </c>
       <c r="F306" s="22" t="str">
         <f>IF(OR(E306="",E306="!!!"),"",IF(NOT(ISNA(VLOOKUP(E306,E$1:E305,1,FALSE()))),"OLD",IF(AND(E306&lt;&gt;"",E306&lt;&gt;"!!!"),"NEW","")))</f>
@@ -13200,7 +13126,7 @@
         <v/>
       </c>
       <c r="L306" s="26" t="s">
-        <v>505</v>
+        <v>476</v>
       </c>
     </row>
     <row r="307" spans="1:12" x14ac:dyDescent="0.3">
@@ -13285,7 +13211,7 @@
         <v>37</v>
       </c>
       <c r="E309" s="21" t="s">
-        <v>464</v>
+        <v>452</v>
       </c>
       <c r="F309" s="22" t="str">
         <f>IF(OR(E309="",E309="!!!"),"",IF(NOT(ISNA(VLOOKUP(E309,E$1:E308,1,FALSE()))),"OLD",IF(AND(E309&lt;&gt;"",E309&lt;&gt;"!!!"),"NEW","")))</f>
@@ -13681,7 +13607,7 @@
         <v>37</v>
       </c>
       <c r="E320" s="21" t="s">
-        <v>465</v>
+        <v>453</v>
       </c>
       <c r="F320" s="22" t="str">
         <f>IF(OR(E320="",E320="!!!"),"",IF(NOT(ISNA(VLOOKUP(E320,E$1:E319,1,FALSE()))),"OLD",IF(AND(E320&lt;&gt;"",E320&lt;&gt;"!!!"),"NEW","")))</f>
@@ -13782,7 +13708,7 @@
         <v>258</v>
       </c>
       <c r="E323" s="21" t="str">
-        <f t="shared" ref="E323:E386" si="10">IF(D323="?OLD","!!!","")</f>
+        <f t="shared" ref="E323:E384" si="10">IF(D323="?OLD","!!!","")</f>
         <v/>
       </c>
       <c r="F323" s="22" t="str">
@@ -13967,7 +13893,7 @@
         <v>37</v>
       </c>
       <c r="E328" s="21" t="s">
-        <v>465</v>
+        <v>453</v>
       </c>
       <c r="F328" s="22" t="str">
         <f>IF(OR(E328="",E328="!!!"),"",IF(NOT(ISNA(VLOOKUP(E328,E$1:E327,1,FALSE()))),"OLD",IF(AND(E328&lt;&gt;"",E328&lt;&gt;"!!!"),"NEW","")))</f>
@@ -14226,7 +14152,7 @@
         <v>54</v>
       </c>
       <c r="E335" s="21" t="s">
-        <v>466</v>
+        <v>454</v>
       </c>
       <c r="F335" s="22" t="str">
         <f>IF(OR(E335="",E335="!!!"),"",IF(NOT(ISNA(VLOOKUP(E335,E$1:E334,1,FALSE()))),"OLD",IF(AND(E335&lt;&gt;"",E335&lt;&gt;"!!!"),"NEW","")))</f>
@@ -14253,7 +14179,7 @@
         <v/>
       </c>
       <c r="L335" s="26" t="s">
-        <v>506</v>
+        <v>477</v>
       </c>
     </row>
     <row r="336" spans="1:12" x14ac:dyDescent="0.3">
@@ -14329,7 +14255,7 @@
         <v/>
       </c>
       <c r="L337" s="26" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
     </row>
     <row r="338" spans="1:12" x14ac:dyDescent="0.3">
@@ -14346,7 +14272,7 @@
         <v>37</v>
       </c>
       <c r="E338" s="21" t="s">
-        <v>464</v>
+        <v>452</v>
       </c>
       <c r="F338" s="22" t="str">
         <f>IF(OR(E338="",E338="!!!"),"",IF(NOT(ISNA(VLOOKUP(E338,E$1:E337,1,FALSE()))),"OLD",IF(AND(E338&lt;&gt;"",E338&lt;&gt;"!!!"),"NEW","")))</f>
@@ -14880,7 +14806,7 @@
         <v>37</v>
       </c>
       <c r="E353" s="21" t="s">
-        <v>466</v>
+        <v>454</v>
       </c>
       <c r="F353" s="22" t="str">
         <f>IF(OR(E353="",E353="!!!"),"",IF(NOT(ISNA(VLOOKUP(E353,E$1:E352,1,FALSE()))),"OLD",IF(AND(E353&lt;&gt;"",E353&lt;&gt;"!!!"),"NEW","")))</f>
@@ -15117,7 +15043,7 @@
         <v/>
       </c>
       <c r="L359" s="26" t="s">
-        <v>467</v>
+        <v>455</v>
       </c>
     </row>
     <row r="360" spans="1:12" x14ac:dyDescent="0.3">
@@ -15282,17 +15208,16 @@
       <c r="C364" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="E364" s="21" t="str">
-        <f t="shared" si="10"/>
-        <v/>
+      <c r="E364" s="21" t="s">
+        <v>491</v>
       </c>
       <c r="F364" s="22" t="str">
         <f>IF(OR(E364="",E364="!!!"),"",IF(NOT(ISNA(VLOOKUP(E364,E$1:E363,1,FALSE()))),"OLD",IF(AND(E364&lt;&gt;"",E364&lt;&gt;"!!!"),"NEW","")))</f>
-        <v/>
+        <v>NEW</v>
       </c>
       <c r="G364" s="23" t="str">
-        <f>IF(OR(E364="",E364="!!!"),"",IF(OR(J364=0,AND(J364=1,K364=1),AND(J364=1,I364="SBJ"),AND(J364=1,I364=0)),"?IN_FOCUS",IF(J364&lt;=2,"?ACTIVATED",IF(J364&lt;&gt;"","?FAMILIAR",IF(F364="NEW",IF(ISNA(VLOOKUP(E364,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v/>
+        <f ca="1">IF(OR(E364="",E364="!!!"),"",IF(OR(J364=0,AND(J364=1,K364=1),AND(J364=1,I364="SBJ"),AND(J364=1,I364=0)),"?IN_FOCUS",IF(J364&lt;=2,"?ACTIVATED",IF(J364&lt;&gt;"","?FAMILIAR",IF(F364="NEW",IF(ISNA(VLOOKUP(E364,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v>?REFERENTIAL</v>
       </c>
       <c r="H364" s="24" t="str">
         <f t="shared" ca="1" si="11"/>
@@ -15310,7 +15235,9 @@
         <f>IF(OR(E364="",E364="!!!",F364="NEW"),"",INDEX(J$1:J363,SUMPRODUCT(MAX(ROW(E$1:E363)*(E364=E$1:E363)))))</f>
         <v/>
       </c>
-      <c r="L364" s="26"/>
+      <c r="L364" s="26" t="s">
+        <v>455</v>
+      </c>
     </row>
     <row r="365" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A365" t="s">
@@ -15428,7 +15355,7 @@
         <v>37</v>
       </c>
       <c r="E368" s="21" t="s">
-        <v>468</v>
+        <v>456</v>
       </c>
       <c r="F368" s="22" t="str">
         <f>IF(OR(E368="",E368="!!!"),"",IF(NOT(ISNA(VLOOKUP(E368,E$1:E367,1,FALSE()))),"OLD",IF(AND(E368&lt;&gt;"",E368&lt;&gt;"!!!"),"NEW","")))</f>
@@ -15529,7 +15456,7 @@
         <v>184</v>
       </c>
       <c r="E371" s="21" t="s">
-        <v>471</v>
+        <v>459</v>
       </c>
       <c r="F371" s="22" t="str">
         <f>IF(OR(E371="",E371="!!!"),"",IF(NOT(ISNA(VLOOKUP(E371,E$1:E370,1,FALSE()))),"OLD",IF(AND(E371&lt;&gt;"",E371&lt;&gt;"!!!"),"NEW","")))</f>
@@ -15556,7 +15483,7 @@
         <v/>
       </c>
       <c r="L371" s="26" t="s">
-        <v>472</v>
+        <v>460</v>
       </c>
     </row>
     <row r="372" spans="1:12" x14ac:dyDescent="0.3">
@@ -15836,7 +15763,7 @@
         <v/>
       </c>
       <c r="L379" s="26" t="s">
-        <v>467</v>
+        <v>455</v>
       </c>
     </row>
     <row r="380" spans="1:12" x14ac:dyDescent="0.3">
@@ -15958,7 +15885,7 @@
         <v>62</v>
       </c>
       <c r="E383" s="21" t="s">
-        <v>460</v>
+        <v>448</v>
       </c>
       <c r="F383" s="22" t="str">
         <f>IF(OR(E383="",E383="!!!"),"",IF(NOT(ISNA(VLOOKUP(E383,E$1:E382,1,FALSE()))),"OLD",IF(AND(E383&lt;&gt;"",E383&lt;&gt;"!!!"),"NEW","")))</f>
@@ -16059,7 +15986,7 @@
         <v/>
       </c>
       <c r="L385" s="26" t="s">
-        <v>470</v>
+        <v>458</v>
       </c>
     </row>
     <row r="386" spans="1:12" x14ac:dyDescent="0.3">
@@ -16098,7 +16025,7 @@
         <v>290</v>
       </c>
       <c r="E387" s="21" t="str">
-        <f t="shared" ref="E387:E450" si="12">IF(D387="?OLD","!!!","")</f>
+        <f t="shared" ref="E387:E404" si="12">IF(D387="?OLD","!!!","")</f>
         <v/>
       </c>
       <c r="F387" s="22" t="str">
@@ -16110,7 +16037,7 @@
         <v/>
       </c>
       <c r="H387" s="24" t="str">
-        <f t="shared" ref="H387:H450" ca="1" si="13">IF(J387&lt;&gt;1,"",IF(I387="SBJ","CB","?"))</f>
+        <f t="shared" ref="H387:H404" ca="1" si="13">IF(J387&lt;&gt;1,"",IF(I387="SBJ","CB","?"))</f>
         <v/>
       </c>
       <c r="I387" s="25" t="str">
@@ -16141,7 +16068,7 @@
         <v>37</v>
       </c>
       <c r="E388" s="21" t="s">
-        <v>469</v>
+        <v>457</v>
       </c>
       <c r="F388" s="22" t="str">
         <f>IF(OR(E388="",E388="!!!"),"",IF(NOT(ISNA(VLOOKUP(E388,E$1:E387,1,FALSE()))),"OLD",IF(AND(E388&lt;&gt;"",E388&lt;&gt;"!!!"),"NEW","")))</f>
@@ -16361,7 +16288,7 @@
         <v>37</v>
       </c>
       <c r="E394" s="21" t="s">
-        <v>475</v>
+        <v>463</v>
       </c>
       <c r="F394" s="22" t="str">
         <f>IF(OR(E394="",E394="!!!"),"",IF(NOT(ISNA(VLOOKUP(E394,E$1:E393,1,FALSE()))),"OLD",IF(AND(E394&lt;&gt;"",E394&lt;&gt;"!!!"),"NEW","")))</f>
@@ -16388,7 +16315,7 @@
         <v/>
       </c>
       <c r="L394" s="26" t="s">
-        <v>479</v>
+        <v>466</v>
       </c>
     </row>
     <row r="395" spans="1:12" x14ac:dyDescent="0.3">
@@ -16439,15 +16366,15 @@
         <v>37</v>
       </c>
       <c r="E396" s="21" t="s">
-        <v>474</v>
+        <v>462</v>
       </c>
       <c r="F396" s="22" t="str">
         <f>IF(OR(E396="",E396="!!!"),"",IF(NOT(ISNA(VLOOKUP(E396,E$1:E395,1,FALSE()))),"OLD",IF(AND(E396&lt;&gt;"",E396&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v>NEW</v>
       </c>
       <c r="G396" s="23" t="str">
         <f ca="1">IF(OR(E396="",E396="!!!"),"",IF(OR(J396=0,AND(J396=1,K396=1),AND(J396=1,I396="SBJ"),AND(J396=1,I396=0)),"?IN_FOCUS",IF(J396&lt;=2,"?ACTIVATED",IF(J396&lt;&gt;"","?FAMILIAR",IF(F396="NEW",IF(ISNA(VLOOKUP(E396,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <v>?REFERENTIAL</v>
       </c>
       <c r="H396" s="24" t="str">
         <f t="shared" ca="1" si="13"/>
@@ -16455,14 +16382,14 @@
       </c>
       <c r="I396" s="25" t="str">
         <f>IF(OR(E396="",E396="!!!",F396="NEW"),"",INDEX(B$2:B395,-1+SUMPRODUCT(MAX(ROW(E$2:E395)*(E396=E$2:E395)))))</f>
-        <v>other_7</v>
-      </c>
-      <c r="J396" s="25">
+        <v/>
+      </c>
+      <c r="J396" s="25" t="str">
         <f ca="1">IF(OR(E396="",E396="!!!",F396="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E396)*(E396=E$2:E396)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E395)*(E2=E$1:E395))))))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K396" s="25" t="str">
-        <f ca="1">IF(OR(E396="",E396="!!!",F396="NEW"),"",INDEX(J$1:J395,SUMPRODUCT(MAX(ROW(E$1:E395)*(E396=E$1:E395)))))</f>
+        <f>IF(OR(E396="",E396="!!!",F396="NEW"),"",INDEX(J$1:J395,SUMPRODUCT(MAX(ROW(E$1:E395)*(E396=E$1:E395)))))</f>
         <v/>
       </c>
       <c r="L396" s="26"/>
@@ -16515,7 +16442,7 @@
         <v>37</v>
       </c>
       <c r="E398" s="21" t="s">
-        <v>461</v>
+        <v>449</v>
       </c>
       <c r="F398" s="22" t="str">
         <f>IF(OR(E398="",E398="!!!"),"",IF(NOT(ISNA(VLOOKUP(E398,E$1:E397,1,FALSE()))),"OLD",IF(AND(E398&lt;&gt;"",E398&lt;&gt;"!!!"),"NEW","")))</f>
@@ -16684,7 +16611,7 @@
         <v/>
       </c>
       <c r="L402" s="26" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
     </row>
     <row r="403" spans="1:12" x14ac:dyDescent="0.3">
@@ -16701,7 +16628,7 @@
         <v>37</v>
       </c>
       <c r="E403" s="21" t="s">
-        <v>473</v>
+        <v>461</v>
       </c>
       <c r="F403" s="22" t="str">
         <f>IF(OR(E403="",E403="!!!"),"",IF(NOT(ISNA(VLOOKUP(E403,E$1:E402,1,FALSE()))),"OLD",IF(AND(E403&lt;&gt;"",E403&lt;&gt;"!!!"),"NEW","")))</f>
@@ -16974,7 +16901,7 @@
         <v/>
       </c>
       <c r="L412" s="26" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
     </row>
     <row r="413" spans="1:12" x14ac:dyDescent="0.3">
@@ -17021,16 +16948,13 @@
       <c r="C414" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="E414" s="21" t="s">
-        <v>508</v>
-      </c>
-      <c r="F414" s="22" t="str">
-        <f>IF(OR(E414="",E414="!!!"),"",IF(NOT(ISNA(VLOOKUP(E414,E$1:E413,1,FALSE()))),"OLD",IF(AND(E414&lt;&gt;"",E414&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>NEW</v>
+      <c r="E414" s="21"/>
+      <c r="F414" s="22" t="s">
+        <v>436</v>
       </c>
       <c r="G414" s="23" t="str">
-        <f ca="1">IF(OR(E414="",E414="!!!"),"",IF(OR(J414=0,AND(J414=1,K414=1),AND(J414=1,I414="SBJ"),AND(J414=1,I414=0)),"?IN_FOCUS",IF(J414&lt;=2,"?ACTIVATED",IF(J414&lt;&gt;"","?FAMILIAR",IF(F414="NEW",IF(ISNA(VLOOKUP(E414,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?REFERENTIAL</v>
+        <f>IF(OR(E414="",E414="!!!"),"",IF(OR(J414=0,AND(J414=1,K414=1),AND(J414=1,I414="SBJ"),AND(J414=1,I414=0)),"?IN_FOCUS",IF(J414&lt;=2,"?ACTIVATED",IF(J414&lt;&gt;"","?FAMILIAR",IF(F414="NEW",IF(ISNA(VLOOKUP(E414,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H414" s="24" t="str">
         <f t="shared" ca="1" si="15"/>
@@ -17048,7 +16972,9 @@
         <f>IF(OR(E414="",E414="!!!",F414="NEW"),"",INDEX(J$1:J413,SUMPRODUCT(MAX(ROW(E$1:E413)*(E414=E$1:E413)))))</f>
         <v/>
       </c>
-      <c r="L414" s="26"/>
+      <c r="L414" s="26" t="s">
+        <v>438</v>
+      </c>
     </row>
     <row r="415" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A415" t="s">
@@ -17372,31 +17298,29 @@
       <c r="C424" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="E424" s="21" t="s">
-        <v>471</v>
-      </c>
+      <c r="E424" s="21"/>
       <c r="F424" s="22" t="str">
         <f>IF(OR(E424="",E424="!!!"),"",IF(NOT(ISNA(VLOOKUP(E424,E$1:E423,1,FALSE()))),"OLD",IF(AND(E424&lt;&gt;"",E424&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v/>
       </c>
       <c r="G424" s="23" t="str">
-        <f ca="1">IF(OR(E424="",E424="!!!"),"",IF(OR(J424=0,AND(J424=1,K424=1),AND(J424=1,I424="SBJ"),AND(J424=1,I424=0)),"?IN_FOCUS",IF(J424&lt;=2,"?ACTIVATED",IF(J424&lt;&gt;"","?FAMILIAR",IF(F424="NEW",IF(ISNA(VLOOKUP(E424,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E424="",E424="!!!"),"",IF(OR(J424=0,AND(J424=1,K424=1),AND(J424=1,I424="SBJ"),AND(J424=1,I424=0)),"?IN_FOCUS",IF(J424&lt;=2,"?ACTIVATED",IF(J424&lt;&gt;"","?FAMILIAR",IF(F424="NEW",IF(ISNA(VLOOKUP(E424,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H424" s="24" t="str">
         <f t="shared" ca="1" si="15"/>
         <v/>
       </c>
-      <c r="I424" s="25">
+      <c r="I424" s="25" t="str">
         <f>IF(OR(E424="",E424="!!!",F424="NEW"),"",INDEX(B$2:B423,-1+SUMPRODUCT(MAX(ROW(E$2:E423)*(E424=E$2:E423)))))</f>
-        <v>0</v>
-      </c>
-      <c r="J424" s="25">
+        <v/>
+      </c>
+      <c r="J424" s="25" t="str">
         <f ca="1">IF(OR(E424="",E424="!!!",F424="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E424)*(E424=E$2:E424)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E423)*(E2=E$1:E423))))))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K424" s="25" t="str">
-        <f ca="1">IF(OR(E424="",E424="!!!",F424="NEW"),"",INDEX(J$1:J423,SUMPRODUCT(MAX(ROW(E$1:E423)*(E424=E$1:E423)))))</f>
+        <f>IF(OR(E424="",E424="!!!",F424="NEW"),"",INDEX(J$1:J423,SUMPRODUCT(MAX(ROW(E$1:E423)*(E424=E$1:E423)))))</f>
         <v/>
       </c>
       <c r="L424" s="26"/>
@@ -17483,10 +17407,10 @@
         <v>37</v>
       </c>
       <c r="E427" s="21" t="s">
-        <v>480</v>
+        <v>467</v>
       </c>
       <c r="F427" s="22" t="s">
-        <v>502</v>
+        <v>475</v>
       </c>
       <c r="G427" s="23" t="str">
         <f ca="1">IF(OR(E427="",E427="!!!"),"",IF(OR(J427=0,AND(J427=1,K427=1),AND(J427=1,I427="SBJ"),AND(J427=1,I427=0)),"?IN_FOCUS",IF(J427&lt;=2,"?ACTIVATED",IF(J427&lt;&gt;"","?FAMILIAR",IF(F427="NEW",IF(ISNA(VLOOKUP(E427,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
@@ -17509,7 +17433,7 @@
         <v/>
       </c>
       <c r="L427" s="26" t="s">
-        <v>507</v>
+        <v>478</v>
       </c>
     </row>
     <row r="428" spans="1:12" x14ac:dyDescent="0.3">
@@ -17733,7 +17657,7 @@
         <v>62</v>
       </c>
       <c r="E434" s="21" t="s">
-        <v>471</v>
+        <v>459</v>
       </c>
       <c r="F434" s="22" t="str">
         <f>IF(OR(E434="",E434="!!!"),"",IF(NOT(ISNA(VLOOKUP(E434,E$1:E433,1,FALSE()))),"OLD",IF(AND(E434&lt;&gt;"",E434&lt;&gt;"!!!"),"NEW","")))</f>
@@ -17747,17 +17671,17 @@
         <f t="shared" ca="1" si="15"/>
         <v/>
       </c>
-      <c r="I434" s="25" t="str">
+      <c r="I434" s="25">
         <f>IF(OR(E434="",E434="!!!",F434="NEW"),"",INDEX(B$2:B433,-1+SUMPRODUCT(MAX(ROW(E$2:E433)*(E434=E$2:E433)))))</f>
-        <v>OBJ_14</v>
+        <v>0</v>
       </c>
       <c r="J434" s="25">
         <f ca="1">IF(OR(E434="",E434="!!!",F434="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E434)*(E434=E$2:E434)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E433)*(E2=E$1:E433))))))</f>
         <v>0</v>
       </c>
-      <c r="K434" s="25">
+      <c r="K434" s="25" t="str">
         <f ca="1">IF(OR(E434="",E434="!!!",F434="NEW"),"",INDEX(J$1:J433,SUMPRODUCT(MAX(ROW(E$1:E433)*(E434=E$1:E433)))))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="L434" s="26"/>
     </row>
@@ -17834,7 +17758,7 @@
         <v/>
       </c>
       <c r="L436" s="26" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
     </row>
     <row r="437" spans="1:12" x14ac:dyDescent="0.3">
@@ -17847,16 +17771,14 @@
       <c r="C437" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="E437" s="21" t="s">
-        <v>492</v>
-      </c>
+      <c r="E437" s="21"/>
       <c r="F437" s="22" t="str">
         <f>IF(OR(E437="",E437="!!!"),"",IF(NOT(ISNA(VLOOKUP(E437,E$1:E436,1,FALSE()))),"OLD",IF(AND(E437&lt;&gt;"",E437&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>NEW</v>
+        <v/>
       </c>
       <c r="G437" s="23" t="str">
-        <f ca="1">IF(OR(E437="",E437="!!!"),"",IF(OR(J437=0,AND(J437=1,K437=1),AND(J437=1,I437="SBJ"),AND(J437=1,I437=0)),"?IN_FOCUS",IF(J437&lt;=2,"?ACTIVATED",IF(J437&lt;&gt;"","?FAMILIAR",IF(F437="NEW",IF(ISNA(VLOOKUP(E437,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?REFERENTIAL</v>
+        <f>IF(OR(E437="",E437="!!!"),"",IF(OR(J437=0,AND(J437=1,K437=1),AND(J437=1,I437="SBJ"),AND(J437=1,I437=0)),"?IN_FOCUS",IF(J437&lt;=2,"?ACTIVATED",IF(J437&lt;&gt;"","?FAMILIAR",IF(F437="NEW",IF(ISNA(VLOOKUP(E437,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H437" s="24" t="str">
         <f t="shared" ca="1" si="15"/>
@@ -17951,16 +17873,14 @@
       <c r="B440" s="20" t="s">
         <v>320</v>
       </c>
-      <c r="E440" s="21" t="s">
-        <v>492</v>
-      </c>
+      <c r="E440" s="21"/>
       <c r="F440" s="22" t="str">
         <f>IF(OR(E440="",E440="!!!"),"",IF(NOT(ISNA(VLOOKUP(E440,E$1:E439,1,FALSE()))),"OLD",IF(AND(E440&lt;&gt;"",E440&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v/>
       </c>
       <c r="G440" s="23" t="str">
-        <f ca="1">IF(OR(E440="",E440="!!!"),"",IF(OR(J440=0,AND(J440=1,K440=1),AND(J440=1,I440="SBJ"),AND(J440=1,I440=0)),"?IN_FOCUS",IF(J440&lt;=2,"?ACTIVATED",IF(J440&lt;&gt;"","?FAMILIAR",IF(F440="NEW",IF(ISNA(VLOOKUP(E440,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E440="",E440="!!!"),"",IF(OR(J440=0,AND(J440=1,K440=1),AND(J440=1,I440="SBJ"),AND(J440=1,I440=0)),"?IN_FOCUS",IF(J440&lt;=2,"?ACTIVATED",IF(J440&lt;&gt;"","?FAMILIAR",IF(F440="NEW",IF(ISNA(VLOOKUP(E440,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H440" s="24" t="str">
         <f t="shared" ca="1" si="15"/>
@@ -17968,14 +17888,14 @@
       </c>
       <c r="I440" s="25" t="str">
         <f>IF(OR(E440="",E440="!!!",F440="NEW"),"",INDEX(B$2:B439,-1+SUMPRODUCT(MAX(ROW(E$2:E439)*(E440=E$2:E439)))))</f>
-        <v>other_12</v>
-      </c>
-      <c r="J440" s="25">
+        <v/>
+      </c>
+      <c r="J440" s="25" t="str">
         <f ca="1">IF(OR(E440="",E440="!!!",F440="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E440)*(E440=E$2:E440)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E439)*(E2=E$1:E439))))))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K440" s="25" t="str">
-        <f ca="1">IF(OR(E440="",E440="!!!",F440="NEW"),"",INDEX(J$1:J439,SUMPRODUCT(MAX(ROW(E$1:E439)*(E440=E$1:E439)))))</f>
+        <f>IF(OR(E440="",E440="!!!",F440="NEW"),"",INDEX(J$1:J439,SUMPRODUCT(MAX(ROW(E$1:E439)*(E440=E$1:E439)))))</f>
         <v/>
       </c>
       <c r="L440" s="26"/>
@@ -18028,15 +17948,15 @@
         <v>37</v>
       </c>
       <c r="E442" s="21" t="s">
-        <v>476</v>
+        <v>464</v>
       </c>
       <c r="F442" s="22" t="str">
         <f>IF(OR(E442="",E442="!!!"),"",IF(NOT(ISNA(VLOOKUP(E442,E$1:E441,1,FALSE()))),"OLD",IF(AND(E442&lt;&gt;"",E442&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v>NEW</v>
       </c>
       <c r="G442" s="23" t="str">
         <f ca="1">IF(OR(E442="",E442="!!!"),"",IF(OR(J442=0,AND(J442=1,K442=1),AND(J442=1,I442="SBJ"),AND(J442=1,I442=0)),"?IN_FOCUS",IF(J442&lt;=2,"?ACTIVATED",IF(J442&lt;&gt;"","?FAMILIAR",IF(F442="NEW",IF(ISNA(VLOOKUP(E442,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <v>?REFERENTIAL</v>
       </c>
       <c r="H442" s="24" t="str">
         <f t="shared" ca="1" si="15"/>
@@ -18044,14 +17964,14 @@
       </c>
       <c r="I442" s="25" t="str">
         <f>IF(OR(E442="",E442="!!!",F442="NEW"),"",INDEX(B$2:B441,-1+SUMPRODUCT(MAX(ROW(E$2:E441)*(E442=E$2:E441)))))</f>
-        <v>OBJ_6</v>
-      </c>
-      <c r="J442" s="25">
+        <v/>
+      </c>
+      <c r="J442" s="25" t="str">
         <f ca="1">IF(OR(E442="",E442="!!!",F442="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E442)*(E442=E$2:E442)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E441)*(E2=E$1:E441))))))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K442" s="25" t="str">
-        <f ca="1">IF(OR(E442="",E442="!!!",F442="NEW"),"",INDEX(J$1:J441,SUMPRODUCT(MAX(ROW(E$1:E441)*(E442=E$1:E441)))))</f>
+        <f>IF(OR(E442="",E442="!!!",F442="NEW"),"",INDEX(J$1:J441,SUMPRODUCT(MAX(ROW(E$1:E441)*(E442=E$1:E441)))))</f>
         <v/>
       </c>
       <c r="L442" s="26"/>
@@ -18060,16 +17980,14 @@
       <c r="A443" t="s">
         <v>328</v>
       </c>
-      <c r="E443" s="21" t="s">
-        <v>477</v>
-      </c>
+      <c r="E443" s="21"/>
       <c r="F443" s="22" t="str">
         <f>IF(OR(E443="",E443="!!!"),"",IF(NOT(ISNA(VLOOKUP(E443,E$1:E442,1,FALSE()))),"OLD",IF(AND(E443&lt;&gt;"",E443&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>NEW</v>
+        <v/>
       </c>
       <c r="G443" s="23" t="str">
-        <f ca="1">IF(OR(E443="",E443="!!!"),"",IF(OR(J443=0,AND(J443=1,K443=1),AND(J443=1,I443="SBJ"),AND(J443=1,I443=0)),"?IN_FOCUS",IF(J443&lt;=2,"?ACTIVATED",IF(J443&lt;&gt;"","?FAMILIAR",IF(F443="NEW",IF(ISNA(VLOOKUP(E443,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?REFERENTIAL</v>
+        <f>IF(OR(E443="",E443="!!!"),"",IF(OR(J443=0,AND(J443=1,K443=1),AND(J443=1,I443="SBJ"),AND(J443=1,I443=0)),"?IN_FOCUS",IF(J443&lt;=2,"?ACTIVATED",IF(J443&lt;&gt;"","?FAMILIAR",IF(F443="NEW",IF(ISNA(VLOOKUP(E443,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H443" s="24" t="str">
         <f t="shared" ca="1" si="15"/>
@@ -18161,31 +18079,29 @@
       <c r="A446" t="s">
         <v>330</v>
       </c>
-      <c r="E446" s="21" t="s">
-        <v>477</v>
-      </c>
+      <c r="E446" s="21"/>
       <c r="F446" s="22" t="str">
         <f>IF(OR(E446="",E446="!!!"),"",IF(NOT(ISNA(VLOOKUP(E446,E$1:E445,1,FALSE()))),"OLD",IF(AND(E446&lt;&gt;"",E446&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v/>
       </c>
       <c r="G446" s="23" t="str">
-        <f ca="1">IF(OR(E446="",E446="!!!"),"",IF(OR(J446=0,AND(J446=1,K446=1),AND(J446=1,I446="SBJ"),AND(J446=1,I446=0)),"?IN_FOCUS",IF(J446&lt;=2,"?ACTIVATED",IF(J446&lt;&gt;"","?FAMILIAR",IF(F446="NEW",IF(ISNA(VLOOKUP(E446,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E446="",E446="!!!"),"",IF(OR(J446=0,AND(J446=1,K446=1),AND(J446=1,I446="SBJ"),AND(J446=1,I446=0)),"?IN_FOCUS",IF(J446&lt;=2,"?ACTIVATED",IF(J446&lt;&gt;"","?FAMILIAR",IF(F446="NEW",IF(ISNA(VLOOKUP(E446,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H446" s="24" t="str">
         <f t="shared" ca="1" si="15"/>
         <v/>
       </c>
-      <c r="I446" s="25">
+      <c r="I446" s="25" t="str">
         <f>IF(OR(E446="",E446="!!!",F446="NEW"),"",INDEX(B$2:B445,-1+SUMPRODUCT(MAX(ROW(E$2:E445)*(E446=E$2:E445)))))</f>
-        <v>0</v>
-      </c>
-      <c r="J446" s="25">
+        <v/>
+      </c>
+      <c r="J446" s="25" t="str">
         <f ca="1">IF(OR(E446="",E446="!!!",F446="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E446)*(E446=E$2:E446)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E445)*(E2=E$1:E445))))))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K446" s="25" t="str">
-        <f ca="1">IF(OR(E446="",E446="!!!",F446="NEW"),"",INDEX(J$1:J445,SUMPRODUCT(MAX(ROW(E$1:E445)*(E446=E$1:E445)))))</f>
+        <f>IF(OR(E446="",E446="!!!",F446="NEW"),"",INDEX(J$1:J445,SUMPRODUCT(MAX(ROW(E$1:E445)*(E446=E$1:E445)))))</f>
         <v/>
       </c>
       <c r="L446" s="26"/>
@@ -18205,7 +18121,7 @@
       </c>
       <c r="E447" s="21"/>
       <c r="F447" s="22" t="s">
-        <v>452</v>
+        <v>442</v>
       </c>
       <c r="G447" s="23" t="str">
         <f>IF(OR(E447="",E447="!!!"),"",IF(OR(J447=0,AND(J447=1,K447=1),AND(J447=1,I447="SBJ"),AND(J447=1,I447=0)),"?IN_FOCUS",IF(J447&lt;=2,"?ACTIVATED",IF(J447&lt;&gt;"","?FAMILIAR",IF(F447="NEW",IF(ISNA(VLOOKUP(E447,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
@@ -18227,9 +18143,7 @@
         <f>IF(OR(E447="",E447="!!!",F447="NEW"),"",INDEX(J$1:J446,SUMPRODUCT(MAX(ROW(E$1:E446)*(E447=E$1:E446)))))</f>
         <v/>
       </c>
-      <c r="L447" s="26" t="s">
-        <v>453</v>
-      </c>
+      <c r="L447" s="26"/>
     </row>
     <row r="448" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A448" t="s">
@@ -18279,7 +18193,7 @@
         <v>37</v>
       </c>
       <c r="E449" s="21" t="s">
-        <v>474</v>
+        <v>462</v>
       </c>
       <c r="F449" s="22" t="str">
         <f>IF(OR(E449="",E449="!!!"),"",IF(NOT(ISNA(VLOOKUP(E449,E$1:E448,1,FALSE()))),"OLD",IF(AND(E449&lt;&gt;"",E449&lt;&gt;"!!!"),"NEW","")))</f>
@@ -18301,9 +18215,9 @@
         <f ca="1">IF(OR(E449="",E449="!!!",F449="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E449)*(E449=E$2:E449)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E448)*(E2=E$1:E448))))))</f>
         <v>0</v>
       </c>
-      <c r="K449" s="25">
+      <c r="K449" s="25" t="str">
         <f ca="1">IF(OR(E449="",E449="!!!",F449="NEW"),"",INDEX(J$1:J448,SUMPRODUCT(MAX(ROW(E$1:E448)*(E449=E$1:E448)))))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="L449" s="26"/>
     </row>
@@ -18355,7 +18269,7 @@
         <v>37</v>
       </c>
       <c r="E451" s="21" t="s">
-        <v>461</v>
+        <v>449</v>
       </c>
       <c r="F451" s="22" t="str">
         <f>IF(OR(E451="",E451="!!!"),"",IF(NOT(ISNA(VLOOKUP(E451,E$1:E450,1,FALSE()))),"OLD",IF(AND(E451&lt;&gt;"",E451&lt;&gt;"!!!"),"NEW","")))</f>
@@ -18524,7 +18438,7 @@
         <v/>
       </c>
       <c r="L455" s="26" t="s">
-        <v>467</v>
+        <v>455</v>
       </c>
     </row>
     <row r="456" spans="1:12" x14ac:dyDescent="0.3">
@@ -18609,7 +18523,7 @@
         <v>37</v>
       </c>
       <c r="E458" s="21" t="s">
-        <v>480</v>
+        <v>467</v>
       </c>
       <c r="F458" s="22" t="str">
         <f>IF(OR(E458="",E458="!!!"),"",IF(NOT(ISNA(VLOOKUP(E458,E$1:E457,1,FALSE()))),"OLD",IF(AND(E458&lt;&gt;"",E458&lt;&gt;"!!!"),"NEW","")))</f>
@@ -18824,7 +18738,7 @@
         <v>62</v>
       </c>
       <c r="E464" s="21" t="s">
-        <v>471</v>
+        <v>459</v>
       </c>
       <c r="F464" s="22" t="str">
         <f>IF(OR(E464="",E464="!!!"),"",IF(NOT(ISNA(VLOOKUP(E464,E$1:E463,1,FALSE()))),"OLD",IF(AND(E464&lt;&gt;"",E464&lt;&gt;"!!!"),"NEW","")))</f>
@@ -19100,16 +19014,14 @@
       <c r="C472" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="E472" s="21" t="s">
-        <v>481</v>
-      </c>
+      <c r="E472" s="21"/>
       <c r="F472" s="22" t="str">
         <f>IF(OR(E472="",E472="!!!"),"",IF(NOT(ISNA(VLOOKUP(E472,E$1:E471,1,FALSE()))),"OLD",IF(AND(E472&lt;&gt;"",E472&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>NEW</v>
+        <v/>
       </c>
       <c r="G472" s="23" t="str">
-        <f ca="1">IF(OR(E472="",E472="!!!"),"",IF(OR(J472=0,AND(J472=1,K472=1),AND(J472=1,I472="SBJ"),AND(J472=1,I472=0)),"?IN_FOCUS",IF(J472&lt;=2,"?ACTIVATED",IF(J472&lt;&gt;"","?FAMILIAR",IF(F472="NEW",IF(ISNA(VLOOKUP(E472,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?REFERENTIAL</v>
+        <f>IF(OR(E472="",E472="!!!"),"",IF(OR(J472=0,AND(J472=1,K472=1),AND(J472=1,I472="SBJ"),AND(J472=1,I472=0)),"?IN_FOCUS",IF(J472&lt;=2,"?ACTIVATED",IF(J472&lt;&gt;"","?FAMILIAR",IF(F472="NEW",IF(ISNA(VLOOKUP(E472,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H472" s="24" t="str">
         <f t="shared" ref="H472:H535" ca="1" si="16">IF(J472&lt;&gt;1,"",IF(I472="SBJ","CB","?"))</f>
@@ -19127,16 +19039,14 @@
         <f>IF(OR(E472="",E472="!!!",F472="NEW"),"",INDEX(J$1:J471,SUMPRODUCT(MAX(ROW(E$1:E471)*(E472=E$1:E471)))))</f>
         <v/>
       </c>
-      <c r="L472" s="26" t="s">
-        <v>428</v>
-      </c>
+      <c r="L472" s="26"/>
     </row>
     <row r="473" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A473" t="s">
         <v>47</v>
       </c>
       <c r="E473" s="21" t="str">
-        <f t="shared" ref="E472:E535" si="17">IF(D473="?OLD","!!!","")</f>
+        <f t="shared" ref="E473:E535" si="17">IF(D473="?OLD","!!!","")</f>
         <v/>
       </c>
       <c r="F473" s="22" t="str">
@@ -19178,16 +19088,14 @@
       <c r="D474" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="E474" s="21" t="s">
-        <v>481</v>
-      </c>
+      <c r="E474" s="21"/>
       <c r="F474" s="22" t="str">
         <f>IF(OR(E474="",E474="!!!"),"",IF(NOT(ISNA(VLOOKUP(E474,E$1:E473,1,FALSE()))),"OLD",IF(AND(E474&lt;&gt;"",E474&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v/>
       </c>
       <c r="G474" s="23" t="str">
-        <f ca="1">IF(OR(E474="",E474="!!!"),"",IF(OR(J474=0,AND(J474=1,K474=1),AND(J474=1,I474="SBJ"),AND(J474=1,I474=0)),"?IN_FOCUS",IF(J474&lt;=2,"?ACTIVATED",IF(J474&lt;&gt;"","?FAMILIAR",IF(F474="NEW",IF(ISNA(VLOOKUP(E474,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E474="",E474="!!!"),"",IF(OR(J474=0,AND(J474=1,K474=1),AND(J474=1,I474="SBJ"),AND(J474=1,I474=0)),"?IN_FOCUS",IF(J474&lt;=2,"?ACTIVATED",IF(J474&lt;&gt;"","?FAMILIAR",IF(F474="NEW",IF(ISNA(VLOOKUP(E474,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H474" s="24" t="str">
         <f t="shared" ca="1" si="16"/>
@@ -19195,14 +19103,14 @@
       </c>
       <c r="I474" s="25" t="str">
         <f>IF(OR(E474="",E474="!!!",F474="NEW"),"",INDEX(B$2:B473,-1+SUMPRODUCT(MAX(ROW(E$2:E473)*(E474=E$2:E473)))))</f>
-        <v>other_9</v>
-      </c>
-      <c r="J474" s="25">
+        <v/>
+      </c>
+      <c r="J474" s="25" t="str">
         <f ca="1">IF(OR(E474="",E474="!!!",F474="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E474)*(E474=E$2:E474)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E473)*(E2=E$1:E473))))))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K474" s="25" t="str">
-        <f ca="1">IF(OR(E474="",E474="!!!",F474="NEW"),"",INDEX(J$1:J473,SUMPRODUCT(MAX(ROW(E$1:E473)*(E474=E$1:E473)))))</f>
+        <f>IF(OR(E474="",E474="!!!",F474="NEW"),"",INDEX(J$1:J473,SUMPRODUCT(MAX(ROW(E$1:E473)*(E474=E$1:E473)))))</f>
         <v/>
       </c>
       <c r="L474" s="26"/>
@@ -19221,7 +19129,7 @@
         <v>37</v>
       </c>
       <c r="E475" s="21" t="s">
-        <v>480</v>
+        <v>467</v>
       </c>
       <c r="F475" s="22" t="str">
         <f>IF(OR(E475="",E475="!!!"),"",IF(NOT(ISNA(VLOOKUP(E475,E$1:E474,1,FALSE()))),"OLD",IF(AND(E475&lt;&gt;"",E475&lt;&gt;"!!!"),"NEW","")))</f>
@@ -19405,7 +19313,7 @@
         <v>37</v>
       </c>
       <c r="E480" s="21" t="s">
-        <v>468</v>
+        <v>456</v>
       </c>
       <c r="F480" s="22" t="str">
         <f>IF(OR(E480="",E480="!!!"),"",IF(NOT(ISNA(VLOOKUP(E480,E$1:E479,1,FALSE()))),"OLD",IF(AND(E480&lt;&gt;"",E480&lt;&gt;"!!!"),"NEW","")))</f>
@@ -19648,7 +19556,7 @@
         <v>54</v>
       </c>
       <c r="E487" s="21" t="s">
-        <v>482</v>
+        <v>468</v>
       </c>
       <c r="F487" s="22" t="str">
         <f>IF(OR(E487="",E487="!!!"),"",IF(NOT(ISNA(VLOOKUP(E487,E$1:E486,1,FALSE()))),"OLD",IF(AND(E487&lt;&gt;"",E487&lt;&gt;"!!!"),"NEW","")))</f>
@@ -19744,7 +19652,7 @@
       </c>
       <c r="L489" s="26"/>
     </row>
-    <row r="490" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="490" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A490" t="s">
         <v>348</v>
       </c>
@@ -19757,14 +19665,15 @@
       <c r="D490" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="E490" s="21"/>
-      <c r="F490" s="22" t="str">
-        <f>IF(OR(E490="",E490="!!!"),"",IF(NOT(ISNA(VLOOKUP(E490,E$1:E489,1,FALSE()))),"OLD",IF(AND(E490&lt;&gt;"",E490&lt;&gt;"!!!"),"NEW","")))</f>
-        <v/>
+      <c r="E490" s="21" t="s">
+        <v>492</v>
+      </c>
+      <c r="F490" s="22" t="s">
+        <v>475</v>
       </c>
       <c r="G490" s="23" t="str">
-        <f>IF(OR(E490="",E490="!!!"),"",IF(OR(J490=0,AND(J490=1,K490=1),AND(J490=1,I490="SBJ"),AND(J490=1,I490=0)),"?IN_FOCUS",IF(J490&lt;=2,"?ACTIVATED",IF(J490&lt;&gt;"","?FAMILIAR",IF(F490="NEW",IF(ISNA(VLOOKUP(E490,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v/>
+        <f ca="1">IF(OR(E490="",E490="!!!"),"",IF(OR(J490=0,AND(J490=1,K490=1),AND(J490=1,I490="SBJ"),AND(J490=1,I490=0)),"?IN_FOCUS",IF(J490&lt;=2,"?ACTIVATED",IF(J490&lt;&gt;"","?FAMILIAR",IF(F490="NEW",IF(ISNA(VLOOKUP(E490,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v>?REFERENTIAL</v>
       </c>
       <c r="H490" s="24" t="str">
         <f t="shared" ca="1" si="16"/>
@@ -19783,7 +19692,7 @@
         <v/>
       </c>
       <c r="L490" s="26" t="s">
-        <v>429</v>
+        <v>493</v>
       </c>
     </row>
     <row r="491" spans="1:12" x14ac:dyDescent="0.3">
@@ -19824,16 +19733,13 @@
       <c r="A492" t="s">
         <v>349</v>
       </c>
-      <c r="E492" s="21" t="s">
-        <v>482</v>
-      </c>
-      <c r="F492" s="22" t="str">
-        <f>IF(OR(E492="",E492="!!!"),"",IF(NOT(ISNA(VLOOKUP(E492,E$1:E491,1,FALSE()))),"OLD",IF(AND(E492&lt;&gt;"",E492&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+      <c r="E492" s="21"/>
+      <c r="F492" s="22" t="s">
+        <v>444</v>
       </c>
       <c r="G492" s="23" t="str">
-        <f ca="1">IF(OR(E492="",E492="!!!"),"",IF(OR(J492=0,AND(J492=1,K492=1),AND(J492=1,I492="SBJ"),AND(J492=1,I492=0)),"?IN_FOCUS",IF(J492&lt;=2,"?ACTIVATED",IF(J492&lt;&gt;"","?FAMILIAR",IF(F492="NEW",IF(ISNA(VLOOKUP(E492,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E492="",E492="!!!"),"",IF(OR(J492=0,AND(J492=1,K492=1),AND(J492=1,I492="SBJ"),AND(J492=1,I492=0)),"?IN_FOCUS",IF(J492&lt;=2,"?ACTIVATED",IF(J492&lt;&gt;"","?FAMILIAR",IF(F492="NEW",IF(ISNA(VLOOKUP(E492,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H492" s="24" t="str">
         <f t="shared" ca="1" si="16"/>
@@ -19841,14 +19747,14 @@
       </c>
       <c r="I492" s="25" t="str">
         <f>IF(OR(E492="",E492="!!!",F492="NEW"),"",INDEX(B$2:B491,-1+SUMPRODUCT(MAX(ROW(E$2:E491)*(E492=E$2:E491)))))</f>
-        <v>OBJ_8</v>
-      </c>
-      <c r="J492" s="25">
+        <v/>
+      </c>
+      <c r="J492" s="25" t="str">
         <f ca="1">IF(OR(E492="",E492="!!!",F492="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E492)*(E492=E$2:E492)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E491)*(E2=E$1:E491))))))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K492" s="25" t="str">
-        <f ca="1">IF(OR(E492="",E492="!!!",F492="NEW"),"",INDEX(J$1:J491,SUMPRODUCT(MAX(ROW(E$1:E491)*(E492=E$1:E491)))))</f>
+        <f>IF(OR(E492="",E492="!!!",F492="NEW"),"",INDEX(J$1:J491,SUMPRODUCT(MAX(ROW(E$1:E491)*(E492=E$1:E491)))))</f>
         <v/>
       </c>
       <c r="L492" s="26"/>
@@ -19900,34 +19806,34 @@
       <c r="D494" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="E494" s="21" t="s">
-        <v>482</v>
-      </c>
+      <c r="E494" s="21"/>
       <c r="F494" s="22" t="str">
         <f>IF(OR(E494="",E494="!!!"),"",IF(NOT(ISNA(VLOOKUP(E494,E$1:E493,1,FALSE()))),"OLD",IF(AND(E494&lt;&gt;"",E494&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v/>
       </c>
       <c r="G494" s="23" t="str">
-        <f ca="1">IF(OR(E494="",E494="!!!"),"",IF(OR(J494=0,AND(J494=1,K494=1),AND(J494=1,I494="SBJ"),AND(J494=1,I494=0)),"?IN_FOCUS",IF(J494&lt;=2,"?ACTIVATED",IF(J494&lt;&gt;"","?FAMILIAR",IF(F494="NEW",IF(ISNA(VLOOKUP(E494,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E494="",E494="!!!"),"",IF(OR(J494=0,AND(J494=1,K494=1),AND(J494=1,I494="SBJ"),AND(J494=1,I494=0)),"?IN_FOCUS",IF(J494&lt;=2,"?ACTIVATED",IF(J494&lt;&gt;"","?FAMILIAR",IF(F494="NEW",IF(ISNA(VLOOKUP(E494,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H494" s="24" t="str">
         <f t="shared" ca="1" si="16"/>
         <v/>
       </c>
-      <c r="I494" s="25">
+      <c r="I494" s="25" t="str">
         <f>IF(OR(E494="",E494="!!!",F494="NEW"),"",INDEX(B$2:B493,-1+SUMPRODUCT(MAX(ROW(E$2:E493)*(E494=E$2:E493)))))</f>
-        <v>0</v>
-      </c>
-      <c r="J494" s="25">
+        <v/>
+      </c>
+      <c r="J494" s="25" t="str">
         <f ca="1">IF(OR(E494="",E494="!!!",F494="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E494)*(E494=E$2:E494)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E493)*(E2=E$1:E493))))))</f>
-        <v>0</v>
-      </c>
-      <c r="K494" s="25">
-        <f ca="1">IF(OR(E494="",E494="!!!",F494="NEW"),"",INDEX(J$1:J493,SUMPRODUCT(MAX(ROW(E$1:E493)*(E494=E$1:E493)))))</f>
-        <v>0</v>
-      </c>
-      <c r="L494" s="26"/>
+        <v/>
+      </c>
+      <c r="K494" s="25" t="str">
+        <f>IF(OR(E494="",E494="!!!",F494="NEW"),"",INDEX(J$1:J493,SUMPRODUCT(MAX(ROW(E$1:E493)*(E494=E$1:E493)))))</f>
+        <v/>
+      </c>
+      <c r="L494" s="26" t="s">
+        <v>504</v>
+      </c>
     </row>
     <row r="495" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A495" t="s">
@@ -20252,7 +20158,7 @@
         <v>62</v>
       </c>
       <c r="E504" s="21" t="s">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="F504" s="22" t="str">
         <f>IF(OR(E504="",E504="!!!"),"",IF(NOT(ISNA(VLOOKUP(E504,E$1:E503,1,FALSE()))),"OLD",IF(AND(E504&lt;&gt;"",E504&lt;&gt;"!!!"),"NEW","")))</f>
@@ -20461,7 +20367,7 @@
         <v>360</v>
       </c>
       <c r="E510" s="21" t="s">
-        <v>480</v>
+        <v>467</v>
       </c>
       <c r="F510" s="22" t="str">
         <f>IF(OR(E510="",E510="!!!"),"",IF(NOT(ISNA(VLOOKUP(E510,E$1:E509,1,FALSE()))),"OLD",IF(AND(E510&lt;&gt;"",E510&lt;&gt;"!!!"),"NEW","")))</f>
@@ -20488,7 +20394,7 @@
         <v>0</v>
       </c>
       <c r="L510" s="26" t="s">
-        <v>509</v>
+        <v>479</v>
       </c>
     </row>
     <row r="511" spans="1:12" x14ac:dyDescent="0.3">
@@ -20525,7 +20431,7 @@
       </c>
       <c r="L511" s="26"/>
     </row>
-    <row r="512" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="512" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A512" t="s">
         <v>175</v>
       </c>
@@ -20536,7 +20442,7 @@
         <v>176</v>
       </c>
       <c r="E512" s="21" t="s">
-        <v>483</v>
+        <v>469</v>
       </c>
       <c r="F512" s="22" t="str">
         <f>IF(OR(E512="",E512="!!!"),"",IF(NOT(ISNA(VLOOKUP(E512,E$1:E511,1,FALSE()))),"OLD",IF(AND(E512&lt;&gt;"",E512&lt;&gt;"!!!"),"NEW","")))</f>
@@ -20563,7 +20469,7 @@
         <v/>
       </c>
       <c r="L512" s="26" t="s">
-        <v>484</v>
+        <v>505</v>
       </c>
     </row>
     <row r="513" spans="1:12" x14ac:dyDescent="0.3">
@@ -20682,7 +20588,7 @@
         <v>37</v>
       </c>
       <c r="E516" s="21" t="s">
-        <v>483</v>
+        <v>469</v>
       </c>
       <c r="F516" s="22" t="str">
         <f>IF(OR(E516="",E516="!!!"),"",IF(NOT(ISNA(VLOOKUP(E516,E$1:E515,1,FALSE()))),"OLD",IF(AND(E516&lt;&gt;"",E516&lt;&gt;"!!!"),"NEW","")))</f>
@@ -21575,33 +21481,31 @@
       <c r="D541" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="E541" s="21" t="s">
-        <v>486</v>
-      </c>
-      <c r="F541" s="22" t="s">
-        <v>485</v>
-      </c>
-      <c r="G541" s="23" t="e">
-        <f ca="1">IF(OR(E541="",E541="!!!"),"",IF(OR(J541=0,AND(J541=1,K541=1),AND(J541=1,I541="SBJ"),AND(J541=1,I541=0)),"?IN_FOCUS",IF(J541&lt;=2,"?ACTIVATED",IF(J541&lt;&gt;"","?FAMILIAR",IF(F541="NEW",IF(ISNA(VLOOKUP(E541,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>#VALUE!</v>
+      <c r="E541" s="21"/>
+      <c r="F541" s="22"/>
+      <c r="G541" s="23" t="str">
+        <f>IF(OR(E541="",E541="!!!"),"",IF(OR(J541=0,AND(J541=1,K541=1),AND(J541=1,I541="SBJ"),AND(J541=1,I541=0)),"?IN_FOCUS",IF(J541&lt;=2,"?ACTIVATED",IF(J541&lt;&gt;"","?FAMILIAR",IF(F541="NEW",IF(ISNA(VLOOKUP(E541,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H541" s="24" t="str">
         <f t="shared" ca="1" si="19"/>
         <v/>
       </c>
-      <c r="I541" s="25" t="e">
+      <c r="I541" s="25" t="str">
         <f>IF(OR(E541="",E541="!!!",F541="NEW"),"",INDEX(B$2:B540,-1+SUMPRODUCT(MAX(ROW(E$2:E540)*(E541=E$2:E540)))))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="J541" s="25">
+        <v/>
+      </c>
+      <c r="J541" s="25" t="str">
         <f ca="1">IF(OR(E541="",E541="!!!",F541="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E541)*(E541=E$2:E541)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E540)*(E2=E$1:E540))))))</f>
-        <v>0</v>
-      </c>
-      <c r="K541" s="25" t="e">
+        <v/>
+      </c>
+      <c r="K541" s="25" t="str">
         <f>IF(OR(E541="",E541="!!!",F541="NEW"),"",INDEX(J$1:J540,SUMPRODUCT(MAX(ROW(E$1:E540)*(E541=E$1:E540)))))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L541" s="26"/>
+        <v/>
+      </c>
+      <c r="L541" s="26" t="s">
+        <v>494</v>
+      </c>
     </row>
     <row r="542" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A542" t="s">
@@ -21749,16 +21653,14 @@
       <c r="C546" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="E546" s="21" t="s">
-        <v>486</v>
-      </c>
+      <c r="E546" s="21"/>
       <c r="F546" s="22" t="str">
         <f>IF(OR(E546="",E546="!!!"),"",IF(NOT(ISNA(VLOOKUP(E546,E$1:E545,1,FALSE()))),"OLD",IF(AND(E546&lt;&gt;"",E546&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v/>
       </c>
       <c r="G546" s="23" t="str">
-        <f ca="1">IF(OR(E546="",E546="!!!"),"",IF(OR(J546=0,AND(J546=1,K546=1),AND(J546=1,I546="SBJ"),AND(J546=1,I546=0)),"?IN_FOCUS",IF(J546&lt;=2,"?ACTIVATED",IF(J546&lt;&gt;"","?FAMILIAR",IF(F546="NEW",IF(ISNA(VLOOKUP(E546,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E546="",E546="!!!"),"",IF(OR(J546=0,AND(J546=1,K546=1),AND(J546=1,I546="SBJ"),AND(J546=1,I546=0)),"?IN_FOCUS",IF(J546&lt;=2,"?ACTIVATED",IF(J546&lt;&gt;"","?FAMILIAR",IF(F546="NEW",IF(ISNA(VLOOKUP(E546,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H546" s="24" t="str">
         <f t="shared" ca="1" si="19"/>
@@ -21766,15 +21668,15 @@
       </c>
       <c r="I546" s="25" t="str">
         <f>IF(OR(E546="",E546="!!!",F546="NEW"),"",INDEX(B$2:B545,-1+SUMPRODUCT(MAX(ROW(E$2:E545)*(E546=E$2:E545)))))</f>
-        <v>other_9</v>
-      </c>
-      <c r="J546" s="25">
+        <v/>
+      </c>
+      <c r="J546" s="25" t="str">
         <f ca="1">IF(OR(E546="",E546="!!!",F546="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E546)*(E546=E$2:E546)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E545)*(E2=E$1:E545))))))</f>
-        <v>0</v>
-      </c>
-      <c r="K546" s="25">
-        <f ca="1">IF(OR(E546="",E546="!!!",F546="NEW"),"",INDEX(J$1:J545,SUMPRODUCT(MAX(ROW(E$1:E545)*(E546=E$1:E545)))))</f>
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="K546" s="25" t="str">
+        <f>IF(OR(E546="",E546="!!!",F546="NEW"),"",INDEX(J$1:J545,SUMPRODUCT(MAX(ROW(E$1:E545)*(E546=E$1:E545)))))</f>
+        <v/>
       </c>
       <c r="L546" s="26"/>
     </row>
@@ -21932,17 +21834,16 @@
       <c r="C551" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="E551" s="21" t="str">
-        <f t="shared" si="18"/>
-        <v/>
+      <c r="E551" s="21" t="s">
+        <v>495</v>
       </c>
       <c r="F551" s="22" t="str">
         <f>IF(OR(E551="",E551="!!!"),"",IF(NOT(ISNA(VLOOKUP(E551,E$1:E550,1,FALSE()))),"OLD",IF(AND(E551&lt;&gt;"",E551&lt;&gt;"!!!"),"NEW","")))</f>
-        <v/>
+        <v>NEW</v>
       </c>
       <c r="G551" s="23" t="str">
-        <f>IF(OR(E551="",E551="!!!"),"",IF(OR(J551=0,AND(J551=1,K551=1),AND(J551=1,I551="SBJ"),AND(J551=1,I551=0)),"?IN_FOCUS",IF(J551&lt;=2,"?ACTIVATED",IF(J551&lt;&gt;"","?FAMILIAR",IF(F551="NEW",IF(ISNA(VLOOKUP(E551,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v/>
+        <f ca="1">IF(OR(E551="",E551="!!!"),"",IF(OR(J551=0,AND(J551=1,K551=1),AND(J551=1,I551="SBJ"),AND(J551=1,I551=0)),"?IN_FOCUS",IF(J551&lt;=2,"?ACTIVATED",IF(J551&lt;&gt;"","?FAMILIAR",IF(F551="NEW",IF(ISNA(VLOOKUP(E551,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v>?REFERENTIAL</v>
       </c>
       <c r="H551" s="24" t="str">
         <f t="shared" ca="1" si="19"/>
@@ -21960,7 +21861,9 @@
         <f>IF(OR(E551="",E551="!!!",F551="NEW"),"",INDEX(J$1:J550,SUMPRODUCT(MAX(ROW(E$1:E550)*(E551=E$1:E550)))))</f>
         <v/>
       </c>
-      <c r="L551" s="26"/>
+      <c r="L551" s="26" t="s">
+        <v>496</v>
+      </c>
     </row>
     <row r="552" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A552" t="s">
@@ -22049,7 +21952,7 @@
         <v>62</v>
       </c>
       <c r="E554" s="21" t="s">
-        <v>466</v>
+        <v>454</v>
       </c>
       <c r="F554" s="22" t="str">
         <f>IF(OR(E554="",E554="!!!"),"",IF(NOT(ISNA(VLOOKUP(E554,E$1:E553,1,FALSE()))),"OLD",IF(AND(E554&lt;&gt;"",E554&lt;&gt;"!!!"),"NEW","")))</f>
@@ -22076,7 +21979,7 @@
         <v>0</v>
       </c>
       <c r="L554" s="26" t="s">
-        <v>497</v>
+        <v>473</v>
       </c>
     </row>
     <row r="555" spans="1:12" x14ac:dyDescent="0.3">
@@ -22117,15 +22020,13 @@
       <c r="A556" t="s">
         <v>204</v>
       </c>
-      <c r="E556" s="21" t="s">
-        <v>466</v>
-      </c>
+      <c r="E556" s="21"/>
       <c r="F556" s="22" t="s">
-        <v>452</v>
+        <v>444</v>
       </c>
       <c r="G556" s="23" t="str">
-        <f ca="1">IF(OR(E556="",E556="!!!"),"",IF(OR(J556=0,AND(J556=1,K556=1),AND(J556=1,I556="SBJ"),AND(J556=1,I556=0)),"?IN_FOCUS",IF(J556&lt;=2,"?ACTIVATED",IF(J556&lt;&gt;"","?FAMILIAR",IF(F556="NEW",IF(ISNA(VLOOKUP(E556,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E556="",E556="!!!"),"",IF(OR(J556=0,AND(J556=1,K556=1),AND(J556=1,I556="SBJ"),AND(J556=1,I556=0)),"?IN_FOCUS",IF(J556&lt;=2,"?ACTIVATED",IF(J556&lt;&gt;"","?FAMILIAR",IF(F556="NEW",IF(ISNA(VLOOKUP(E556,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H556" s="24" t="str">
         <f t="shared" ca="1" si="19"/>
@@ -22133,19 +22034,17 @@
       </c>
       <c r="I556" s="25" t="str">
         <f>IF(OR(E556="",E556="!!!",F556="NEW"),"",INDEX(B$2:B555,-1+SUMPRODUCT(MAX(ROW(E$2:E555)*(E556=E$2:E555)))))</f>
-        <v>other_6</v>
-      </c>
-      <c r="J556" s="25">
+        <v/>
+      </c>
+      <c r="J556" s="25" t="str">
         <f ca="1">IF(OR(E556="",E556="!!!",F556="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E556)*(E556=E$2:E556)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E555)*(E2=E$1:E555))))))</f>
-        <v>0</v>
-      </c>
-      <c r="K556" s="25">
-        <f ca="1">IF(OR(E556="",E556="!!!",F556="NEW"),"",INDEX(J$1:J555,SUMPRODUCT(MAX(ROW(E$1:E555)*(E556=E$1:E555)))))</f>
-        <v>0</v>
-      </c>
-      <c r="L556" s="26" t="s">
-        <v>487</v>
-      </c>
+        <v/>
+      </c>
+      <c r="K556" s="25" t="str">
+        <f>IF(OR(E556="",E556="!!!",F556="NEW"),"",INDEX(J$1:J555,SUMPRODUCT(MAX(ROW(E$1:E555)*(E556=E$1:E555)))))</f>
+        <v/>
+      </c>
+      <c r="L556" s="26"/>
     </row>
     <row r="557" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A557" t="s">
@@ -22263,7 +22162,7 @@
         <v>37</v>
       </c>
       <c r="E560" s="21" t="s">
-        <v>488</v>
+        <v>497</v>
       </c>
       <c r="F560" s="22" t="str">
         <f>IF(OR(E560="",E560="!!!"),"",IF(NOT(ISNA(VLOOKUP(E560,E$1:E559,1,FALSE()))),"OLD",IF(AND(E560&lt;&gt;"",E560&lt;&gt;"!!!"),"NEW","")))</f>
@@ -22335,16 +22234,14 @@
       <c r="C562" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="E562" s="21" t="s">
-        <v>489</v>
-      </c>
+      <c r="E562" s="21"/>
       <c r="F562" s="22" t="str">
         <f>IF(OR(E562="",E562="!!!"),"",IF(NOT(ISNA(VLOOKUP(E562,E$1:E561,1,FALSE()))),"OLD",IF(AND(E562&lt;&gt;"",E562&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>NEW</v>
+        <v/>
       </c>
       <c r="G562" s="23" t="str">
-        <f ca="1">IF(OR(E562="",E562="!!!"),"",IF(OR(J562=0,AND(J562=1,K562=1),AND(J562=1,I562="SBJ"),AND(J562=1,I562=0)),"?IN_FOCUS",IF(J562&lt;=2,"?ACTIVATED",IF(J562&lt;&gt;"","?FAMILIAR",IF(F562="NEW",IF(ISNA(VLOOKUP(E562,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?REFERENTIAL</v>
+        <f>IF(OR(E562="",E562="!!!"),"",IF(OR(J562=0,AND(J562=1,K562=1),AND(J562=1,I562="SBJ"),AND(J562=1,I562=0)),"?IN_FOCUS",IF(J562&lt;=2,"?ACTIVATED",IF(J562&lt;&gt;"","?FAMILIAR",IF(F562="NEW",IF(ISNA(VLOOKUP(E562,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H562" s="24" t="str">
         <f t="shared" ca="1" si="19"/>
@@ -22405,16 +22302,14 @@
       <c r="B564" s="20" t="s">
         <v>386</v>
       </c>
-      <c r="E564" s="21" t="s">
-        <v>490</v>
-      </c>
+      <c r="E564" s="21"/>
       <c r="F564" s="22" t="str">
         <f>IF(OR(E564="",E564="!!!"),"",IF(NOT(ISNA(VLOOKUP(E564,E$1:E563,1,FALSE()))),"OLD",IF(AND(E564&lt;&gt;"",E564&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>NEW</v>
+        <v/>
       </c>
       <c r="G564" s="23" t="str">
-        <f ca="1">IF(OR(E564="",E564="!!!"),"",IF(OR(J564=0,AND(J564=1,K564=1),AND(J564=1,I564="SBJ"),AND(J564=1,I564=0)),"?IN_FOCUS",IF(J564&lt;=2,"?ACTIVATED",IF(J564&lt;&gt;"","?FAMILIAR",IF(F564="NEW",IF(ISNA(VLOOKUP(E564,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?REFERENTIAL</v>
+        <f>IF(OR(E564="",E564="!!!"),"",IF(OR(J564=0,AND(J564=1,K564=1),AND(J564=1,I564="SBJ"),AND(J564=1,I564=0)),"?IN_FOCUS",IF(J564&lt;=2,"?ACTIVATED",IF(J564&lt;&gt;"","?FAMILIAR",IF(F564="NEW",IF(ISNA(VLOOKUP(E564,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H564" s="24" t="str">
         <f t="shared" ca="1" si="19"/>
@@ -22448,7 +22343,7 @@
         <v>37</v>
       </c>
       <c r="E565" s="21" t="s">
-        <v>480</v>
+        <v>467</v>
       </c>
       <c r="F565" s="22" t="str">
         <f>IF(OR(E565="",E565="!!!"),"",IF(NOT(ISNA(VLOOKUP(E565,E$1:E564,1,FALSE()))),"OLD",IF(AND(E565&lt;&gt;"",E565&lt;&gt;"!!!"),"NEW","")))</f>
@@ -22524,7 +22419,7 @@
         <v>37</v>
       </c>
       <c r="E567" s="21" t="s">
-        <v>480</v>
+        <v>467</v>
       </c>
       <c r="F567" s="22" t="str">
         <f>IF(OR(E567="",E567="!!!"),"",IF(NOT(ISNA(VLOOKUP(E567,E$1:E566,1,FALSE()))),"OLD",IF(AND(E567&lt;&gt;"",E567&lt;&gt;"!!!"),"NEW","")))</f>
@@ -22562,17 +22457,16 @@
       <c r="C568" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="E568" s="21" t="str">
-        <f t="shared" si="18"/>
-        <v/>
+      <c r="E568" s="21" t="s">
+        <v>498</v>
       </c>
       <c r="F568" s="22" t="str">
         <f>IF(OR(E568="",E568="!!!"),"",IF(NOT(ISNA(VLOOKUP(E568,E$1:E567,1,FALSE()))),"OLD",IF(AND(E568&lt;&gt;"",E568&lt;&gt;"!!!"),"NEW","")))</f>
-        <v/>
+        <v>NEW</v>
       </c>
       <c r="G568" s="23" t="str">
-        <f>IF(OR(E568="",E568="!!!"),"",IF(OR(J568=0,AND(J568=1,K568=1),AND(J568=1,I568="SBJ"),AND(J568=1,I568=0)),"?IN_FOCUS",IF(J568&lt;=2,"?ACTIVATED",IF(J568&lt;&gt;"","?FAMILIAR",IF(F568="NEW",IF(ISNA(VLOOKUP(E568,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v/>
+        <f ca="1">IF(OR(E568="",E568="!!!"),"",IF(OR(J568=0,AND(J568=1,K568=1),AND(J568=1,I568="SBJ"),AND(J568=1,I568=0)),"?IN_FOCUS",IF(J568&lt;=2,"?ACTIVATED",IF(J568&lt;&gt;"","?FAMILIAR",IF(F568="NEW",IF(ISNA(VLOOKUP(E568,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v>?REFERENTIAL</v>
       </c>
       <c r="H568" s="24" t="str">
         <f t="shared" ca="1" si="19"/>
@@ -22590,7 +22484,9 @@
         <f>IF(OR(E568="",E568="!!!",F568="NEW"),"",INDEX(J$1:J567,SUMPRODUCT(MAX(ROW(E$1:E567)*(E568=E$1:E567)))))</f>
         <v/>
       </c>
-      <c r="L568" s="26"/>
+      <c r="L568" s="26" t="s">
+        <v>496</v>
+      </c>
     </row>
     <row r="569" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A569" t="s">
@@ -22875,7 +22771,7 @@
         <v>62</v>
       </c>
       <c r="E577" s="21" t="s">
-        <v>483</v>
+        <v>469</v>
       </c>
       <c r="F577" s="22" t="str">
         <f>IF(OR(E577="",E577="!!!"),"",IF(NOT(ISNA(VLOOKUP(E577,E$1:E576,1,FALSE()))),"OLD",IF(AND(E577&lt;&gt;"",E577&lt;&gt;"!!!"),"NEW","")))</f>
@@ -22902,7 +22798,7 @@
         <v>0</v>
       </c>
       <c r="L577" s="26" t="s">
-        <v>510</v>
+        <v>480</v>
       </c>
     </row>
     <row r="578" spans="1:12" x14ac:dyDescent="0.3">
@@ -23012,7 +22908,7 @@
         <v>154</v>
       </c>
       <c r="E581" s="21" t="s">
-        <v>446</v>
+        <v>437</v>
       </c>
       <c r="F581" s="22" t="str">
         <f>IF(OR(E581="",E581="!!!"),"",IF(NOT(ISNA(VLOOKUP(E581,E$1:E580,1,FALSE()))),"OLD",IF(AND(E581&lt;&gt;"",E581&lt;&gt;"!!!"),"NEW","")))</f>
@@ -23081,32 +22977,30 @@
       <c r="B583" s="20" t="s">
         <v>379</v>
       </c>
-      <c r="E583" s="21" t="s">
-        <v>446</v>
-      </c>
+      <c r="E583" s="21"/>
       <c r="F583" s="22" t="str">
         <f>IF(OR(E583="",E583="!!!"),"",IF(NOT(ISNA(VLOOKUP(E583,E$1:E582,1,FALSE()))),"OLD",IF(AND(E583&lt;&gt;"",E583&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v/>
       </c>
       <c r="G583" s="23" t="str">
-        <f ca="1">IF(OR(E583="",E583="!!!"),"",IF(OR(J583=0,AND(J583=1,K583=1),AND(J583=1,I583="SBJ"),AND(J583=1,I583=0)),"?IN_FOCUS",IF(J583&lt;=2,"?ACTIVATED",IF(J583&lt;&gt;"","?FAMILIAR",IF(F583="NEW",IF(ISNA(VLOOKUP(E583,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E583="",E583="!!!"),"",IF(OR(J583=0,AND(J583=1,K583=1),AND(J583=1,I583="SBJ"),AND(J583=1,I583=0)),"?IN_FOCUS",IF(J583&lt;=2,"?ACTIVATED",IF(J583&lt;&gt;"","?FAMILIAR",IF(F583="NEW",IF(ISNA(VLOOKUP(E583,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H583" s="24" t="str">
         <f t="shared" ca="1" si="19"/>
         <v/>
       </c>
-      <c r="I583" s="25">
+      <c r="I583" s="25" t="str">
         <f>IF(OR(E583="",E583="!!!",F583="NEW"),"",INDEX(B$2:B582,-1+SUMPRODUCT(MAX(ROW(E$2:E582)*(E583=E$2:E582)))))</f>
-        <v>0</v>
-      </c>
-      <c r="J583" s="25">
+        <v/>
+      </c>
+      <c r="J583" s="25" t="str">
         <f ca="1">IF(OR(E583="",E583="!!!",F583="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E583)*(E583=E$2:E583)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E582)*(E2=E$1:E582))))))</f>
-        <v>0</v>
-      </c>
-      <c r="K583" s="25">
-        <f ca="1">IF(OR(E583="",E583="!!!",F583="NEW"),"",INDEX(J$1:J582,SUMPRODUCT(MAX(ROW(E$1:E582)*(E583=E$1:E582)))))</f>
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="K583" s="25" t="str">
+        <f>IF(OR(E583="",E583="!!!",F583="NEW"),"",INDEX(J$1:J582,SUMPRODUCT(MAX(ROW(E$1:E582)*(E583=E$1:E582)))))</f>
+        <v/>
       </c>
       <c r="L583" s="26"/>
     </row>
@@ -23124,7 +23018,7 @@
         <v>37</v>
       </c>
       <c r="E584" s="21" t="s">
-        <v>483</v>
+        <v>469</v>
       </c>
       <c r="F584" s="22" t="str">
         <f>IF(OR(E584="",E584="!!!"),"",IF(NOT(ISNA(VLOOKUP(E584,E$1:E583,1,FALSE()))),"OLD",IF(AND(E584&lt;&gt;"",E584&lt;&gt;"!!!"),"NEW","")))</f>
@@ -23345,7 +23239,7 @@
       </c>
       <c r="E590" s="21"/>
       <c r="F590" s="22" t="s">
-        <v>452</v>
+        <v>442</v>
       </c>
       <c r="G590" s="23" t="str">
         <f>IF(OR(E590="",E590="!!!"),"",IF(OR(J590=0,AND(J590=1,K590=1),AND(J590=1,I590="SBJ"),AND(J590=1,I590=0)),"?IN_FOCUS",IF(J590&lt;=2,"?ACTIVATED",IF(J590&lt;&gt;"","?FAMILIAR",IF(F590="NEW",IF(ISNA(VLOOKUP(E590,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
@@ -23367,9 +23261,7 @@
         <f>IF(OR(E590="",E590="!!!",F590="NEW"),"",INDEX(J$1:J589,SUMPRODUCT(MAX(ROW(E$1:E589)*(E590=E$1:E589)))))</f>
         <v/>
       </c>
-      <c r="L590" s="26" t="s">
-        <v>491</v>
-      </c>
+      <c r="L590" s="26"/>
     </row>
     <row r="591" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A591" t="s">
@@ -23560,14 +23452,16 @@
       <c r="D596" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="E596" s="21"/>
+      <c r="E596" s="21" t="s">
+        <v>499</v>
+      </c>
       <c r="F596" s="22" t="str">
         <f>IF(OR(E596="",E596="!!!"),"",IF(NOT(ISNA(VLOOKUP(E596,E$1:E595,1,FALSE()))),"OLD",IF(AND(E596&lt;&gt;"",E596&lt;&gt;"!!!"),"NEW","")))</f>
-        <v/>
+        <v>NEW</v>
       </c>
       <c r="G596" s="23" t="str">
-        <f>IF(OR(E596="",E596="!!!"),"",IF(OR(J596=0,AND(J596=1,K596=1),AND(J596=1,I596="SBJ"),AND(J596=1,I596=0)),"?IN_FOCUS",IF(J596&lt;=2,"?ACTIVATED",IF(J596&lt;&gt;"","?FAMILIAR",IF(F596="NEW",IF(ISNA(VLOOKUP(E596,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v/>
+        <f ca="1">IF(OR(E596="",E596="!!!"),"",IF(OR(J596=0,AND(J596=1,K596=1),AND(J596=1,I596="SBJ"),AND(J596=1,I596=0)),"?IN_FOCUS",IF(J596&lt;=2,"?ACTIVATED",IF(J596&lt;&gt;"","?FAMILIAR",IF(F596="NEW",IF(ISNA(VLOOKUP(E596,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v>?REFERENTIAL</v>
       </c>
       <c r="H596" s="24" t="str">
         <f t="shared" ca="1" si="19"/>
@@ -23586,7 +23480,7 @@
         <v/>
       </c>
       <c r="L596" s="26" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
     </row>
     <row r="597" spans="1:12" x14ac:dyDescent="0.3">
@@ -23594,30 +23488,30 @@
         <v>395</v>
       </c>
       <c r="E597" s="21" t="s">
-        <v>494</v>
+        <v>437</v>
       </c>
       <c r="F597" s="22" t="s">
-        <v>485</v>
-      </c>
-      <c r="G597" s="23" t="e">
+        <v>433</v>
+      </c>
+      <c r="G597" s="23" t="str">
         <f ca="1">IF(OR(E597="",E597="!!!"),"",IF(OR(J597=0,AND(J597=1,K597=1),AND(J597=1,I597="SBJ"),AND(J597=1,I597=0)),"?IN_FOCUS",IF(J597&lt;=2,"?ACTIVATED",IF(J597&lt;&gt;"","?FAMILIAR",IF(F597="NEW",IF(ISNA(VLOOKUP(E597,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>#VALUE!</v>
+        <v>?IN_FOCUS</v>
       </c>
       <c r="H597" s="24" t="str">
         <f t="shared" ca="1" si="19"/>
         <v/>
       </c>
-      <c r="I597" s="25" t="e">
+      <c r="I597" s="25">
         <f>IF(OR(E597="",E597="!!!",F597="NEW"),"",INDEX(B$2:B596,-1+SUMPRODUCT(MAX(ROW(E$2:E596)*(E597=E$2:E596)))))</f>
-        <v>#VALUE!</v>
+        <v>0</v>
       </c>
       <c r="J597" s="25">
         <f ca="1">IF(OR(E597="",E597="!!!",F597="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E597)*(E597=E$2:E597)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E596)*(E2=E$1:E596))))))</f>
         <v>0</v>
       </c>
-      <c r="K597" s="25" t="e">
-        <f>IF(OR(E597="",E597="!!!",F597="NEW"),"",INDEX(J$1:J596,SUMPRODUCT(MAX(ROW(E$1:E596)*(E597=E$1:E596)))))</f>
-        <v>#VALUE!</v>
+      <c r="K597" s="25">
+        <f ca="1">IF(OR(E597="",E597="!!!",F597="NEW"),"",INDEX(J$1:J596,SUMPRODUCT(MAX(ROW(E$1:E596)*(E597=E$1:E596)))))</f>
+        <v>0</v>
       </c>
       <c r="L597" s="26"/>
     </row>
@@ -23694,7 +23588,7 @@
         <v>47</v>
       </c>
       <c r="E600" s="21" t="str">
-        <f t="shared" ref="E600:E663" si="20">IF(D600="?OLD","!!!","")</f>
+        <f t="shared" ref="E600:E648" si="20">IF(D600="?OLD","!!!","")</f>
         <v/>
       </c>
       <c r="F600" s="22" t="str">
@@ -23706,7 +23600,7 @@
         <v/>
       </c>
       <c r="H600" s="24" t="str">
-        <f t="shared" ref="H600:H663" ca="1" si="21">IF(J600&lt;&gt;1,"",IF(I600="SBJ","CB","?"))</f>
+        <f t="shared" ref="H600:H648" ca="1" si="21">IF(J600&lt;&gt;1,"",IF(I600="SBJ","CB","?"))</f>
         <v/>
       </c>
       <c r="I600" s="25" t="str">
@@ -23730,32 +23624,30 @@
       <c r="B601" s="20" t="s">
         <v>180</v>
       </c>
-      <c r="E601" s="21" t="s">
-        <v>494</v>
-      </c>
+      <c r="E601" s="21"/>
       <c r="F601" s="22" t="str">
         <f>IF(OR(E601="",E601="!!!"),"",IF(NOT(ISNA(VLOOKUP(E601,E$1:E600,1,FALSE()))),"OLD",IF(AND(E601&lt;&gt;"",E601&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+        <v/>
       </c>
       <c r="G601" s="23" t="str">
-        <f ca="1">IF(OR(E601="",E601="!!!"),"",IF(OR(J601=0,AND(J601=1,K601=1),AND(J601=1,I601="SBJ"),AND(J601=1,I601=0)),"?IN_FOCUS",IF(J601&lt;=2,"?ACTIVATED",IF(J601&lt;&gt;"","?FAMILIAR",IF(F601="NEW",IF(ISNA(VLOOKUP(E601,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E601="",E601="!!!"),"",IF(OR(J601=0,AND(J601=1,K601=1),AND(J601=1,I601="SBJ"),AND(J601=1,I601=0)),"?IN_FOCUS",IF(J601&lt;=2,"?ACTIVATED",IF(J601&lt;&gt;"","?FAMILIAR",IF(F601="NEW",IF(ISNA(VLOOKUP(E601,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H601" s="24" t="str">
         <f t="shared" ca="1" si="21"/>
         <v/>
       </c>
-      <c r="I601" s="25">
+      <c r="I601" s="25" t="str">
         <f>IF(OR(E601="",E601="!!!",F601="NEW"),"",INDEX(B$2:B600,-1+SUMPRODUCT(MAX(ROW(E$2:E600)*(E601=E$2:E600)))))</f>
-        <v>0</v>
-      </c>
-      <c r="J601" s="25">
+        <v/>
+      </c>
+      <c r="J601" s="25" t="str">
         <f ca="1">IF(OR(E601="",E601="!!!",F601="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E601)*(E601=E$2:E601)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E600)*(E2=E$1:E600))))))</f>
-        <v>0</v>
-      </c>
-      <c r="K601" s="25">
-        <f ca="1">IF(OR(E601="",E601="!!!",F601="NEW"),"",INDEX(J$1:J600,SUMPRODUCT(MAX(ROW(E$1:E600)*(E601=E$1:E600)))))</f>
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="K601" s="25" t="str">
+        <f>IF(OR(E601="",E601="!!!",F601="NEW"),"",INDEX(J$1:J600,SUMPRODUCT(MAX(ROW(E$1:E600)*(E601=E$1:E600)))))</f>
+        <v/>
       </c>
       <c r="L601" s="26"/>
     </row>
@@ -23840,16 +23732,13 @@
       <c r="D604" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="E604" s="21" t="s">
-        <v>441</v>
-      </c>
-      <c r="F604" s="22" t="str">
-        <f>IF(OR(E604="",E604="!!!"),"",IF(NOT(ISNA(VLOOKUP(E604,E$1:E603,1,FALSE()))),"OLD",IF(AND(E604&lt;&gt;"",E604&lt;&gt;"!!!"),"NEW","")))</f>
-        <v>OLD</v>
+      <c r="E604" s="21"/>
+      <c r="F604" s="22" t="s">
+        <v>436</v>
       </c>
       <c r="G604" s="23" t="str">
-        <f ca="1">IF(OR(E604="",E604="!!!"),"",IF(OR(J604=0,AND(J604=1,K604=1),AND(J604=1,I604="SBJ"),AND(J604=1,I604=0)),"?IN_FOCUS",IF(J604&lt;=2,"?ACTIVATED",IF(J604&lt;&gt;"","?FAMILIAR",IF(F604="NEW",IF(ISNA(VLOOKUP(E604,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v>?IN_FOCUS</v>
+        <f>IF(OR(E604="",E604="!!!"),"",IF(OR(J604=0,AND(J604=1,K604=1),AND(J604=1,I604="SBJ"),AND(J604=1,I604=0)),"?IN_FOCUS",IF(J604&lt;=2,"?ACTIVATED",IF(J604&lt;&gt;"","?FAMILIAR",IF(F604="NEW",IF(ISNA(VLOOKUP(E604,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v/>
       </c>
       <c r="H604" s="24" t="str">
         <f t="shared" ca="1" si="21"/>
@@ -23857,14 +23746,14 @@
       </c>
       <c r="I604" s="25" t="str">
         <f>IF(OR(E604="",E604="!!!",F604="NEW"),"",INDEX(B$2:B603,-1+SUMPRODUCT(MAX(ROW(E$2:E603)*(E604=E$2:E603)))))</f>
-        <v>other</v>
-      </c>
-      <c r="J604" s="25">
+        <v/>
+      </c>
+      <c r="J604" s="25" t="str">
         <f ca="1">IF(OR(E604="",E604="!!!",F604="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E604)*(E604=E$2:E604)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E603)*(E2=E$1:E603))))))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K604" s="25" t="str">
-        <f ca="1">IF(OR(E604="",E604="!!!",F604="NEW"),"",INDEX(J$1:J603,SUMPRODUCT(MAX(ROW(E$1:E603)*(E604=E$1:E603)))))</f>
+        <f>IF(OR(E604="",E604="!!!",F604="NEW"),"",INDEX(J$1:J603,SUMPRODUCT(MAX(ROW(E$1:E603)*(E604=E$1:E603)))))</f>
         <v/>
       </c>
       <c r="L604" s="26"/>
@@ -24336,7 +24225,7 @@
         <v>174</v>
       </c>
       <c r="E618" s="21" t="s">
-        <v>494</v>
+        <v>449</v>
       </c>
       <c r="F618" s="22" t="str">
         <f>IF(OR(E618="",E618="!!!"),"",IF(NOT(ISNA(VLOOKUP(E618,E$1:E617,1,FALSE()))),"OLD",IF(AND(E618&lt;&gt;"",E618&lt;&gt;"!!!"),"NEW","")))</f>
@@ -24352,7 +24241,7 @@
       </c>
       <c r="I618" s="25" t="str">
         <f>IF(OR(E618="",E618="!!!",F618="NEW"),"",INDEX(B$2:B617,-1+SUMPRODUCT(MAX(ROW(E$2:E617)*(E618=E$2:E617)))))</f>
-        <v>SBJ_6</v>
+        <v>other_14</v>
       </c>
       <c r="J618" s="25">
         <f ca="1">IF(OR(E618="",E618="!!!",F618="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E618)*(E618=E$2:E618)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E617)*(E2=E$1:E617))))))</f>
@@ -24374,17 +24263,16 @@
       <c r="C619" s="20" t="s">
         <v>176</v>
       </c>
-      <c r="E619" s="21" t="str">
-        <f t="shared" si="20"/>
-        <v/>
+      <c r="E619" s="21" t="s">
+        <v>462</v>
       </c>
       <c r="F619" s="22" t="str">
         <f>IF(OR(E619="",E619="!!!"),"",IF(NOT(ISNA(VLOOKUP(E619,E$1:E618,1,FALSE()))),"OLD",IF(AND(E619&lt;&gt;"",E619&lt;&gt;"!!!"),"NEW","")))</f>
-        <v/>
+        <v>OLD</v>
       </c>
       <c r="G619" s="23" t="str">
-        <f>IF(OR(E619="",E619="!!!"),"",IF(OR(J619=0,AND(J619=1,K619=1),AND(J619=1,I619="SBJ"),AND(J619=1,I619=0)),"?IN_FOCUS",IF(J619&lt;=2,"?ACTIVATED",IF(J619&lt;&gt;"","?FAMILIAR",IF(F619="NEW",IF(ISNA(VLOOKUP(E619,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v/>
+        <f ca="1">IF(OR(E619="",E619="!!!"),"",IF(OR(J619=0,AND(J619=1,K619=1),AND(J619=1,I619="SBJ"),AND(J619=1,I619=0)),"?IN_FOCUS",IF(J619&lt;=2,"?ACTIVATED",IF(J619&lt;&gt;"","?FAMILIAR",IF(F619="NEW",IF(ISNA(VLOOKUP(E619,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v>?IN_FOCUS</v>
       </c>
       <c r="H619" s="24" t="str">
         <f t="shared" ca="1" si="21"/>
@@ -24392,24 +24280,26 @@
       </c>
       <c r="I619" s="25" t="str">
         <f>IF(OR(E619="",E619="!!!",F619="NEW"),"",INDEX(B$2:B618,-1+SUMPRODUCT(MAX(ROW(E$2:E618)*(E619=E$2:E618)))))</f>
-        <v/>
-      </c>
-      <c r="J619" s="25" t="str">
+        <v>OBJ_13</v>
+      </c>
+      <c r="J619" s="25">
         <f ca="1">IF(OR(E619="",E619="!!!",F619="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E619)*(E619=E$2:E619)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E618)*(E2=E$1:E618))))))</f>
-        <v/>
-      </c>
-      <c r="K619" s="25" t="str">
-        <f>IF(OR(E619="",E619="!!!",F619="NEW"),"",INDEX(J$1:J618,SUMPRODUCT(MAX(ROW(E$1:E618)*(E619=E$1:E618)))))</f>
-        <v/>
-      </c>
-      <c r="L619" s="26"/>
+        <v>0</v>
+      </c>
+      <c r="K619" s="25">
+        <f ca="1">IF(OR(E619="",E619="!!!",F619="NEW"),"",INDEX(J$1:J618,SUMPRODUCT(MAX(ROW(E$1:E618)*(E619=E$1:E618)))))</f>
+        <v>0</v>
+      </c>
+      <c r="L619" s="26" t="s">
+        <v>496</v>
+      </c>
     </row>
     <row r="620" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A620" t="s">
         <v>226</v>
       </c>
       <c r="E620" s="21" t="s">
-        <v>496</v>
+        <v>472</v>
       </c>
       <c r="F620" s="22" t="str">
         <f>IF(OR(E620="",E620="!!!"),"",IF(NOT(ISNA(VLOOKUP(E620,E$1:E619,1,FALSE()))),"OLD",IF(AND(E620&lt;&gt;"",E620&lt;&gt;"!!!"),"NEW","")))</f>
@@ -24436,7 +24326,7 @@
         <v/>
       </c>
       <c r="L620" s="26" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
     </row>
     <row r="621" spans="1:12" x14ac:dyDescent="0.3">
@@ -24512,7 +24402,7 @@
         <v/>
       </c>
       <c r="L622" s="26" t="s">
-        <v>467</v>
+        <v>455</v>
       </c>
     </row>
     <row r="623" spans="1:12" x14ac:dyDescent="0.3">
@@ -24707,7 +24597,7 @@
         <v>37</v>
       </c>
       <c r="E628" s="21" t="s">
-        <v>495</v>
+        <v>471</v>
       </c>
       <c r="F628" s="22" t="str">
         <f>IF(OR(E628="",E628="!!!"),"",IF(NOT(ISNA(VLOOKUP(E628,E$1:E627,1,FALSE()))),"OLD",IF(AND(E628&lt;&gt;"",E628&lt;&gt;"!!!"),"NEW","")))</f>
@@ -24927,7 +24817,7 @@
         <v>37</v>
       </c>
       <c r="E634" s="21" t="s">
-        <v>496</v>
+        <v>472</v>
       </c>
       <c r="F634" s="22" t="str">
         <f>IF(OR(E634="",E634="!!!"),"",IF(NOT(ISNA(VLOOKUP(E634,E$1:E633,1,FALSE()))),"OLD",IF(AND(E634&lt;&gt;"",E634&lt;&gt;"!!!"),"NEW","")))</f>
@@ -25027,16 +24917,15 @@
       <c r="A637" t="s">
         <v>410</v>
       </c>
-      <c r="E637" s="21" t="str">
-        <f t="shared" si="20"/>
-        <v/>
+      <c r="E637" s="21" t="s">
+        <v>462</v>
       </c>
       <c r="F637" s="22" t="s">
-        <v>444</v>
+        <v>433</v>
       </c>
       <c r="G637" s="23" t="str">
-        <f>IF(OR(E637="",E637="!!!"),"",IF(OR(J637=0,AND(J637=1,K637=1),AND(J637=1,I637="SBJ"),AND(J637=1,I637=0)),"?IN_FOCUS",IF(J637&lt;=2,"?ACTIVATED",IF(J637&lt;&gt;"","?FAMILIAR",IF(F637="NEW",IF(ISNA(VLOOKUP(E637,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v/>
+        <f ca="1">IF(OR(E637="",E637="!!!"),"",IF(OR(J637=0,AND(J637=1,K637=1),AND(J637=1,I637="SBJ"),AND(J637=1,I637=0)),"?IN_FOCUS",IF(J637&lt;=2,"?ACTIVATED",IF(J637&lt;&gt;"","?FAMILIAR",IF(F637="NEW",IF(ISNA(VLOOKUP(E637,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v>?IN_FOCUS</v>
       </c>
       <c r="H637" s="24" t="str">
         <f t="shared" ca="1" si="21"/>
@@ -25044,19 +24933,17 @@
       </c>
       <c r="I637" s="25" t="str">
         <f>IF(OR(E637="",E637="!!!",F637="NEW"),"",INDEX(B$2:B636,-1+SUMPRODUCT(MAX(ROW(E$2:E636)*(E637=E$2:E636)))))</f>
-        <v/>
-      </c>
-      <c r="J637" s="25" t="str">
+        <v>other_2</v>
+      </c>
+      <c r="J637" s="25">
         <f ca="1">IF(OR(E637="",E637="!!!",F637="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E637)*(E637=E$2:E637)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E636)*(E2=E$1:E636))))))</f>
-        <v/>
-      </c>
-      <c r="K637" s="25" t="str">
-        <f>IF(OR(E637="",E637="!!!",F637="NEW"),"",INDEX(J$1:J636,SUMPRODUCT(MAX(ROW(E$1:E636)*(E637=E$1:E636)))))</f>
-        <v/>
-      </c>
-      <c r="L637" s="26" t="s">
-        <v>511</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K637" s="25">
+        <f ca="1">IF(OR(E637="",E637="!!!",F637="NEW"),"",INDEX(J$1:J636,SUMPRODUCT(MAX(ROW(E$1:E636)*(E637=E$1:E636)))))</f>
+        <v>0</v>
+      </c>
+      <c r="L637" s="26"/>
     </row>
     <row r="638" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A638" t="s">
@@ -25068,17 +24955,16 @@
       <c r="C638" s="20" t="s">
         <v>176</v>
       </c>
-      <c r="E638" s="21" t="str">
-        <f t="shared" si="20"/>
-        <v/>
+      <c r="E638" s="21" t="s">
+        <v>503</v>
       </c>
       <c r="F638" s="22" t="str">
         <f>IF(OR(E638="",E638="!!!"),"",IF(NOT(ISNA(VLOOKUP(E638,E$1:E637,1,FALSE()))),"OLD",IF(AND(E638&lt;&gt;"",E638&lt;&gt;"!!!"),"NEW","")))</f>
-        <v/>
+        <v>NEW</v>
       </c>
       <c r="G638" s="23" t="str">
-        <f>IF(OR(E638="",E638="!!!"),"",IF(OR(J638=0,AND(J638=1,K638=1),AND(J638=1,I638="SBJ"),AND(J638=1,I638=0)),"?IN_FOCUS",IF(J638&lt;=2,"?ACTIVATED",IF(J638&lt;&gt;"","?FAMILIAR",IF(F638="NEW",IF(ISNA(VLOOKUP(E638,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
-        <v/>
+        <f ca="1">IF(OR(E638="",E638="!!!"),"",IF(OR(J638=0,AND(J638=1,K638=1),AND(J638=1,I638="SBJ"),AND(J638=1,I638=0)),"?IN_FOCUS",IF(J638&lt;=2,"?ACTIVATED",IF(J638&lt;&gt;"","?FAMILIAR",IF(F638="NEW",IF(ISNA(VLOOKUP(E638,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
+        <v>?REFERENTIAL</v>
       </c>
       <c r="H638" s="24" t="str">
         <f t="shared" ca="1" si="21"/>

</xml_diff>